<commit_message>
Consolidate outstanding MethodMesh modules and documentation
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/nfc/example_odk_nfc_credential_provisioning.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/nfc/example_odk_nfc_credential_provisioning.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R828160c944ce4db7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R58c58b8e51054869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R52263252442148fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rdd4766b1ab16440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R06fac21d64274738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Redd2dec1f6a34994"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -266,17 +266,17 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="40" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="120" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="95" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -316,6 +316,7 @@
       <x:c r="L1" s="4" t="str">
         <x:v>body::intent</x:v>
       </x:c>
+      <x:c r="M1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
@@ -324,16 +325,17 @@
       <x:c r="B2" s="8" t="str">
         <x:v>start</x:v>
       </x:c>
-      <x:c r="C2" s="8" t="str"/>
-      <x:c r="D2" s="8" t="str"/>
-      <x:c r="E2" s="8" t="str"/>
-      <x:c r="F2" s="8" t="str"/>
-      <x:c r="G2" s="8" t="str"/>
-      <x:c r="H2" s="8" t="str"/>
-      <x:c r="I2" s="8" t="str"/>
-      <x:c r="J2" s="8" t="str"/>
-      <x:c r="K2" s="8" t="str"/>
-      <x:c r="L2" s="8" t="str"/>
+      <x:c r="C2" s="8"/>
+      <x:c r="D2" s="8"/>
+      <x:c r="E2" s="8"/>
+      <x:c r="F2" s="8"/>
+      <x:c r="G2" s="8"/>
+      <x:c r="H2" s="8"/>
+      <x:c r="I2" s="8"/>
+      <x:c r="J2" s="8"/>
+      <x:c r="K2" s="8"/>
+      <x:c r="L2" s="8"/>
+      <x:c r="M2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -342,16 +344,17 @@
       <x:c r="B3" s="8" t="str">
         <x:v>end</x:v>
       </x:c>
-      <x:c r="C3" s="8" t="str"/>
-      <x:c r="D3" s="8" t="str"/>
-      <x:c r="E3" s="8" t="str"/>
-      <x:c r="F3" s="8" t="str"/>
-      <x:c r="G3" s="8" t="str"/>
-      <x:c r="H3" s="8" t="str"/>
-      <x:c r="I3" s="8" t="str"/>
-      <x:c r="J3" s="8" t="str"/>
-      <x:c r="K3" s="8" t="str"/>
-      <x:c r="L3" s="8" t="str"/>
+      <x:c r="C3" s="8"/>
+      <x:c r="D3" s="8"/>
+      <x:c r="E3" s="8"/>
+      <x:c r="F3" s="8"/>
+      <x:c r="G3" s="8"/>
+      <x:c r="H3" s="8"/>
+      <x:c r="I3" s="8"/>
+      <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
+      <x:c r="L3" s="8"/>
+      <x:c r="M3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="8" t="str">
@@ -364,16 +367,17 @@
         <x:v>Provision a MethodMesh NFC credential</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str">
-        <x:v>Study identity and governance remain in ODK. MethodMesh writes only the portable cryptographic credential and returns the issuer identity and audit evidence.</x:v>
-      </x:c>
-      <x:c r="E4" s="8" t="str"/>
-      <x:c r="F4" s="8" t="str"/>
-      <x:c r="G4" s="8" t="str"/>
-      <x:c r="H4" s="8" t="str"/>
-      <x:c r="I4" s="8" t="str"/>
-      <x:c r="J4" s="8" t="str"/>
-      <x:c r="K4" s="8" t="str"/>
-      <x:c r="L4" s="8" t="str"/>
+        <x:v>This example models a real study credential registry. Personal/study identity is stored in this ODK submission (and later central study systems), while MethodMesh handles the NFC cryptographic credential and returns the actual provisioning-device issuer identity.</x:v>
+      </x:c>
+      <x:c r="E4" s="8"/>
+      <x:c r="F4" s="8"/>
+      <x:c r="G4" s="8"/>
+      <x:c r="H4" s="8"/>
+      <x:c r="I4" s="8"/>
+      <x:c r="J4" s="8"/>
+      <x:c r="K4" s="8"/>
+      <x:c r="L4" s="8"/>
+      <x:c r="M4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
@@ -385,17 +389,18 @@
       <x:c r="C5" s="8" t="str">
         <x:v>Credential holder and study context</x:v>
       </x:c>
-      <x:c r="D5" s="8" t="str"/>
-      <x:c r="E5" s="8" t="str"/>
-      <x:c r="F5" s="8" t="str"/>
-      <x:c r="G5" s="8" t="str"/>
-      <x:c r="H5" s="8" t="str"/>
-      <x:c r="I5" s="8" t="str"/>
+      <x:c r="D5" s="8"/>
+      <x:c r="E5" s="8"/>
+      <x:c r="F5" s="8"/>
+      <x:c r="G5" s="8"/>
+      <x:c r="H5" s="8"/>
+      <x:c r="I5" s="8"/>
       <x:c r="J5" s="8" t="str">
         <x:v>field-list</x:v>
       </x:c>
-      <x:c r="K5" s="8" t="str"/>
-      <x:c r="L5" s="8" t="str"/>
+      <x:c r="K5" s="8"/>
+      <x:c r="L5" s="8"/>
+      <x:c r="M5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
@@ -413,17 +418,18 @@
       <x:c r="E6" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F6" s="8" t="str"/>
+      <x:c r="F6" s="8"/>
       <x:c r="G6" s="8" t="str">
         <x:v>string-length(.) &lt;= 64</x:v>
       </x:c>
       <x:c r="H6" s="8" t="str">
         <x:v>Use a study ID of 64 characters or fewer.</x:v>
       </x:c>
-      <x:c r="I6" s="8" t="str"/>
-      <x:c r="J6" s="8" t="str"/>
-      <x:c r="K6" s="8" t="str"/>
-      <x:c r="L6" s="8" t="str"/>
+      <x:c r="I6" s="8"/>
+      <x:c r="J6" s="8"/>
+      <x:c r="K6" s="8"/>
+      <x:c r="L6" s="8"/>
+      <x:c r="M6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8" t="str">
@@ -435,17 +441,18 @@
       <x:c r="C7" s="8" t="str">
         <x:v>Credential holder type</x:v>
       </x:c>
-      <x:c r="D7" s="8" t="str"/>
+      <x:c r="D7" s="8"/>
       <x:c r="E7" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F7" s="8" t="str"/>
-      <x:c r="G7" s="8" t="str"/>
-      <x:c r="H7" s="8" t="str"/>
-      <x:c r="I7" s="8" t="str"/>
-      <x:c r="J7" s="8" t="str"/>
-      <x:c r="K7" s="8" t="str"/>
-      <x:c r="L7" s="8" t="str"/>
+      <x:c r="F7" s="8"/>
+      <x:c r="G7" s="8"/>
+      <x:c r="H7" s="8"/>
+      <x:c r="I7" s="8"/>
+      <x:c r="J7" s="8"/>
+      <x:c r="K7" s="8"/>
+      <x:c r="L7" s="8"/>
+      <x:c r="M7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8" t="str">
@@ -458,22 +465,23 @@
         <x:v>Credential subject / registry ID</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
-        <x:v>Use a stable pseudonymous ID, not a name or email. This is the identifier passed into the portable credential.</x:v>
+        <x:v>Use a short stable pseudonymous ID, not the person's name or email. This is passed to MethodMesh and recovered after successful PIN verification.</x:v>
       </x:c>
       <x:c r="E8" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F8" s="8" t="str"/>
+      <x:c r="F8" s="8"/>
       <x:c r="G8" s="8" t="str">
         <x:v>string-length(.) &gt;= 2 and string-length(.) &lt;= 64</x:v>
       </x:c>
       <x:c r="H8" s="8" t="str">
         <x:v>Use a stable ID between 2 and 64 characters.</x:v>
       </x:c>
-      <x:c r="I8" s="8" t="str"/>
-      <x:c r="J8" s="8" t="str"/>
-      <x:c r="K8" s="8" t="str"/>
-      <x:c r="L8" s="8" t="str"/>
+      <x:c r="I8" s="8"/>
+      <x:c r="J8" s="8"/>
+      <x:c r="K8" s="8"/>
+      <x:c r="L8" s="8"/>
+      <x:c r="M8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8" t="str">
@@ -486,18 +494,19 @@
         <x:v>Name / display name</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
-        <x:v>Registry field only; not written to the NFC credential.</x:v>
+        <x:v>Registry field only: retained in ODK/Sentinel and not sent to MethodMesh or written to the card.</x:v>
       </x:c>
       <x:c r="E9" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F9" s="8" t="str"/>
-      <x:c r="G9" s="8" t="str"/>
-      <x:c r="H9" s="8" t="str"/>
-      <x:c r="I9" s="8" t="str"/>
-      <x:c r="J9" s="8" t="str"/>
-      <x:c r="K9" s="8" t="str"/>
-      <x:c r="L9" s="8" t="str"/>
+      <x:c r="F9" s="8"/>
+      <x:c r="G9" s="8"/>
+      <x:c r="H9" s="8"/>
+      <x:c r="I9" s="8"/>
+      <x:c r="J9" s="8"/>
+      <x:c r="K9" s="8"/>
+      <x:c r="L9" s="8"/>
+      <x:c r="M9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
@@ -509,17 +518,18 @@
       <x:c r="C10" s="8" t="str">
         <x:v>Study role</x:v>
       </x:c>
-      <x:c r="D10" s="8" t="str"/>
+      <x:c r="D10" s="8"/>
       <x:c r="E10" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F10" s="8" t="str"/>
-      <x:c r="G10" s="8" t="str"/>
-      <x:c r="H10" s="8" t="str"/>
-      <x:c r="I10" s="8" t="str"/>
-      <x:c r="J10" s="8" t="str"/>
-      <x:c r="K10" s="8" t="str"/>
-      <x:c r="L10" s="8" t="str"/>
+      <x:c r="F10" s="8"/>
+      <x:c r="G10" s="8"/>
+      <x:c r="H10" s="8"/>
+      <x:c r="I10" s="8"/>
+      <x:c r="J10" s="8"/>
+      <x:c r="K10" s="8"/>
+      <x:c r="L10" s="8"/>
+      <x:c r="M10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
@@ -531,19 +541,20 @@
       <x:c r="C11" s="8" t="str">
         <x:v>Other role</x:v>
       </x:c>
-      <x:c r="D11" s="8" t="str"/>
+      <x:c r="D11" s="8"/>
       <x:c r="E11" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="F11" s="8" t="str">
         <x:v>${holder_role} = 'other'</x:v>
       </x:c>
-      <x:c r="G11" s="8" t="str"/>
-      <x:c r="H11" s="8" t="str"/>
-      <x:c r="I11" s="8" t="str"/>
-      <x:c r="J11" s="8" t="str"/>
-      <x:c r="K11" s="8" t="str"/>
-      <x:c r="L11" s="8" t="str"/>
+      <x:c r="G11" s="8"/>
+      <x:c r="H11" s="8"/>
+      <x:c r="I11" s="8"/>
+      <x:c r="J11" s="8"/>
+      <x:c r="K11" s="8"/>
+      <x:c r="L11" s="8"/>
+      <x:c r="M11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
@@ -561,13 +572,14 @@
       <x:c r="E12" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F12" s="8" t="str"/>
-      <x:c r="G12" s="8" t="str"/>
-      <x:c r="H12" s="8" t="str"/>
-      <x:c r="I12" s="8" t="str"/>
-      <x:c r="J12" s="8" t="str"/>
-      <x:c r="K12" s="8" t="str"/>
-      <x:c r="L12" s="8" t="str"/>
+      <x:c r="F12" s="8"/>
+      <x:c r="G12" s="8"/>
+      <x:c r="H12" s="8"/>
+      <x:c r="I12" s="8"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="8"/>
+      <x:c r="L12" s="8"/>
+      <x:c r="M12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
@@ -582,14 +594,15 @@
       <x:c r="D13" s="8" t="str">
         <x:v>Optional employing organisation or study team.</x:v>
       </x:c>
-      <x:c r="E13" s="8" t="str"/>
-      <x:c r="F13" s="8" t="str"/>
-      <x:c r="G13" s="8" t="str"/>
-      <x:c r="H13" s="8" t="str"/>
-      <x:c r="I13" s="8" t="str"/>
-      <x:c r="J13" s="8" t="str"/>
-      <x:c r="K13" s="8" t="str"/>
-      <x:c r="L13" s="8" t="str"/>
+      <x:c r="E13" s="8"/>
+      <x:c r="F13" s="8"/>
+      <x:c r="G13" s="8"/>
+      <x:c r="H13" s="8"/>
+      <x:c r="I13" s="8"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="8"/>
+      <x:c r="L13" s="8"/>
+      <x:c r="M13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
@@ -602,18 +615,19 @@
         <x:v>Credential valid from</x:v>
       </x:c>
       <x:c r="D14" s="8" t="str">
-        <x:v>Administrative validity retained by the study registry; not encoded into ROSC1.</x:v>
+        <x:v>Governance/registry validity start. Under the current ROSC1 contract this date is not encoded into the NFC credential itself.</x:v>
       </x:c>
       <x:c r="E14" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F14" s="8" t="str"/>
-      <x:c r="G14" s="8" t="str"/>
-      <x:c r="H14" s="8" t="str"/>
-      <x:c r="I14" s="8" t="str"/>
-      <x:c r="J14" s="8" t="str"/>
-      <x:c r="K14" s="8" t="str"/>
-      <x:c r="L14" s="8" t="str"/>
+      <x:c r="F14" s="8"/>
+      <x:c r="G14" s="8"/>
+      <x:c r="H14" s="8"/>
+      <x:c r="I14" s="8"/>
+      <x:c r="J14" s="8"/>
+      <x:c r="K14" s="8"/>
+      <x:c r="L14" s="8"/>
+      <x:c r="M14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
@@ -626,22 +640,23 @@
         <x:v>Credential valid until</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
-        <x:v>Administrative validity retained by the study registry; not encoded into ROSC1.</x:v>
+        <x:v>Governance/registry validity end. Under the current ROSC1 contract this date is not encoded into the NFC credential itself.</x:v>
       </x:c>
       <x:c r="E15" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F15" s="8" t="str"/>
+      <x:c r="F15" s="8"/>
       <x:c r="G15" s="8" t="str">
         <x:v>. &gt;= ${valid_from_date}</x:v>
       </x:c>
       <x:c r="H15" s="8" t="str">
         <x:v>End date must be on or after the start date.</x:v>
       </x:c>
-      <x:c r="I15" s="8" t="str"/>
-      <x:c r="J15" s="8" t="str"/>
-      <x:c r="K15" s="8" t="str"/>
-      <x:c r="L15" s="8" t="str"/>
+      <x:c r="I15" s="8"/>
+      <x:c r="J15" s="8"/>
+      <x:c r="K15" s="8"/>
+      <x:c r="L15" s="8"/>
+      <x:c r="M15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
@@ -659,13 +674,14 @@
       <x:c r="E16" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F16" s="8" t="str"/>
-      <x:c r="G16" s="8" t="str"/>
-      <x:c r="H16" s="8" t="str"/>
-      <x:c r="I16" s="8" t="str"/>
-      <x:c r="J16" s="8" t="str"/>
-      <x:c r="K16" s="8" t="str"/>
-      <x:c r="L16" s="8" t="str"/>
+      <x:c r="F16" s="8"/>
+      <x:c r="G16" s="8"/>
+      <x:c r="H16" s="8"/>
+      <x:c r="I16" s="8"/>
+      <x:c r="J16" s="8"/>
+      <x:c r="K16" s="8"/>
+      <x:c r="L16" s="8"/>
+      <x:c r="M16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
@@ -677,17 +693,18 @@
       <x:c r="C17" s="8" t="str">
         <x:v>Reason for issuing credential</x:v>
       </x:c>
-      <x:c r="D17" s="8" t="str"/>
+      <x:c r="D17" s="8"/>
       <x:c r="E17" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F17" s="8" t="str"/>
-      <x:c r="G17" s="8" t="str"/>
-      <x:c r="H17" s="8" t="str"/>
-      <x:c r="I17" s="8" t="str"/>
-      <x:c r="J17" s="8" t="str"/>
-      <x:c r="K17" s="8" t="str"/>
-      <x:c r="L17" s="8" t="str"/>
+      <x:c r="F17" s="8"/>
+      <x:c r="G17" s="8"/>
+      <x:c r="H17" s="8"/>
+      <x:c r="I17" s="8"/>
+      <x:c r="J17" s="8"/>
+      <x:c r="K17" s="8"/>
+      <x:c r="L17" s="8"/>
+      <x:c r="M17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
@@ -699,19 +716,20 @@
       <x:c r="C18" s="8" t="str">
         <x:v>Other issuance reason</x:v>
       </x:c>
-      <x:c r="D18" s="8" t="str"/>
+      <x:c r="D18" s="8"/>
       <x:c r="E18" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="F18" s="8" t="str">
         <x:v>${provision_reason} = 'other'</x:v>
       </x:c>
-      <x:c r="G18" s="8" t="str"/>
-      <x:c r="H18" s="8" t="str"/>
-      <x:c r="I18" s="8" t="str"/>
-      <x:c r="J18" s="8" t="str"/>
-      <x:c r="K18" s="8" t="str"/>
-      <x:c r="L18" s="8" t="str"/>
+      <x:c r="G18" s="8"/>
+      <x:c r="H18" s="8"/>
+      <x:c r="I18" s="8"/>
+      <x:c r="J18" s="8"/>
+      <x:c r="K18" s="8"/>
+      <x:c r="L18" s="8"/>
+      <x:c r="M18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
@@ -726,16 +744,17 @@
       <x:c r="D19" s="8" t="str">
         <x:v>Optional study administration notes. Do not enter the PIN.</x:v>
       </x:c>
-      <x:c r="E19" s="8" t="str"/>
-      <x:c r="F19" s="8" t="str"/>
-      <x:c r="G19" s="8" t="str"/>
-      <x:c r="H19" s="8" t="str"/>
-      <x:c r="I19" s="8" t="str"/>
+      <x:c r="E19" s="8"/>
+      <x:c r="F19" s="8"/>
+      <x:c r="G19" s="8"/>
+      <x:c r="H19" s="8"/>
+      <x:c r="I19" s="8"/>
       <x:c r="J19" s="8" t="str">
         <x:v>multiline</x:v>
       </x:c>
-      <x:c r="K19" s="8" t="str"/>
-      <x:c r="L19" s="8" t="str"/>
+      <x:c r="K19" s="8"/>
+      <x:c r="L19" s="8"/>
+      <x:c r="M19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
@@ -744,18 +763,19 @@
       <x:c r="B20" s="8" t="str">
         <x:v>credential_registry_key</x:v>
       </x:c>
-      <x:c r="C20" s="8" t="str"/>
-      <x:c r="D20" s="8" t="str"/>
-      <x:c r="E20" s="8" t="str"/>
-      <x:c r="F20" s="8" t="str"/>
-      <x:c r="G20" s="8" t="str"/>
-      <x:c r="H20" s="8" t="str"/>
+      <x:c r="C20" s="8"/>
+      <x:c r="D20" s="8"/>
+      <x:c r="E20" s="8"/>
+      <x:c r="F20" s="8"/>
+      <x:c r="G20" s="8"/>
+      <x:c r="H20" s="8"/>
       <x:c r="I20" s="8" t="str">
         <x:v>concat(${study_id}, '|', ${credential_subject_id_input})</x:v>
       </x:c>
-      <x:c r="J20" s="8" t="str"/>
-      <x:c r="K20" s="8" t="str"/>
-      <x:c r="L20" s="8" t="str"/>
+      <x:c r="J20" s="8"/>
+      <x:c r="K20" s="8"/>
+      <x:c r="L20" s="8"/>
+      <x:c r="M20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8" t="str">
@@ -764,16 +784,17 @@
       <x:c r="B21" s="8" t="str">
         <x:v>study_context_end</x:v>
       </x:c>
-      <x:c r="C21" s="8" t="str"/>
-      <x:c r="D21" s="8" t="str"/>
-      <x:c r="E21" s="8" t="str"/>
-      <x:c r="F21" s="8" t="str"/>
-      <x:c r="G21" s="8" t="str"/>
-      <x:c r="H21" s="8" t="str"/>
-      <x:c r="I21" s="8" t="str"/>
-      <x:c r="J21" s="8" t="str"/>
-      <x:c r="K21" s="8" t="str"/>
-      <x:c r="L21" s="8" t="str"/>
+      <x:c r="C21" s="8"/>
+      <x:c r="D21" s="8"/>
+      <x:c r="E21" s="8"/>
+      <x:c r="F21" s="8"/>
+      <x:c r="G21" s="8"/>
+      <x:c r="H21" s="8"/>
+      <x:c r="I21" s="8"/>
+      <x:c r="J21" s="8"/>
+      <x:c r="K21" s="8"/>
+      <x:c r="L21" s="8"/>
+      <x:c r="M21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8" t="str">
@@ -785,17 +806,18 @@
       <x:c r="C22" s="8" t="str">
         <x:v>Credential security options</x:v>
       </x:c>
-      <x:c r="D22" s="8" t="str"/>
-      <x:c r="E22" s="8" t="str"/>
-      <x:c r="F22" s="8" t="str"/>
-      <x:c r="G22" s="8" t="str"/>
-      <x:c r="H22" s="8" t="str"/>
-      <x:c r="I22" s="8" t="str"/>
+      <x:c r="D22" s="8"/>
+      <x:c r="E22" s="8"/>
+      <x:c r="F22" s="8"/>
+      <x:c r="G22" s="8"/>
+      <x:c r="H22" s="8"/>
+      <x:c r="I22" s="8"/>
       <x:c r="J22" s="8" t="str">
         <x:v>field-list</x:v>
       </x:c>
-      <x:c r="K22" s="8" t="str"/>
-      <x:c r="L22" s="8" t="str"/>
+      <x:c r="K22" s="8"/>
+      <x:c r="L22" s="8"/>
+      <x:c r="M22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="8" t="str">
@@ -808,20 +830,21 @@
         <x:v>PIN length</x:v>
       </x:c>
       <x:c r="D23" s="8" t="str">
-        <x:v>The PIN is entered only inside MethodMesh.</x:v>
+        <x:v>The PIN itself is entered only inside MethodMesh and is never returned to ODK.</x:v>
       </x:c>
       <x:c r="E23" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F23" s="8" t="str"/>
-      <x:c r="G23" s="8" t="str"/>
-      <x:c r="H23" s="8" t="str"/>
-      <x:c r="I23" s="8" t="str"/>
-      <x:c r="J23" s="8" t="str"/>
+      <x:c r="F23" s="8"/>
+      <x:c r="G23" s="8"/>
+      <x:c r="H23" s="8"/>
+      <x:c r="I23" s="8"/>
+      <x:c r="J23" s="8"/>
       <x:c r="K23" s="8" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="L23" s="8" t="str"/>
+      <x:c r="L23" s="8"/>
+      <x:c r="M23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="8" t="str">
@@ -831,23 +854,24 @@
         <x:v>overwrite_policy_input</x:v>
       </x:c>
       <x:c r="C24" s="8" t="str">
-        <x:v>Existing card content</x:v>
+        <x:v>NFC overwrite policy</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>Use empty_only for new cards. Use replace only when intentionally replacing an existing credential.</x:v>
+        <x:v>Use empty_only for new cards. Replace should only be used when intentionally reissuing/replacing a credential.</x:v>
       </x:c>
       <x:c r="E24" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F24" s="8" t="str"/>
-      <x:c r="G24" s="8" t="str"/>
-      <x:c r="H24" s="8" t="str"/>
-      <x:c r="I24" s="8" t="str"/>
-      <x:c r="J24" s="8" t="str"/>
+      <x:c r="F24" s="8"/>
+      <x:c r="G24" s="8"/>
+      <x:c r="H24" s="8"/>
+      <x:c r="I24" s="8"/>
+      <x:c r="J24" s="8"/>
       <x:c r="K24" s="8" t="str">
         <x:v>empty_only</x:v>
       </x:c>
-      <x:c r="L24" s="8" t="str"/>
+      <x:c r="L24" s="8"/>
+      <x:c r="M24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="8" t="str">
@@ -857,19 +881,20 @@
         <x:v>security_note</x:v>
       </x:c>
       <x:c r="C25" s="8" t="str">
-        <x:v>PIN and issuer-key handling</x:v>
+        <x:v>PIN and credential secret handling</x:v>
       </x:c>
       <x:c r="D25" s="8" t="str">
-        <x:v>The PIN and private issuer key never return to ODK. The private signing key remains in Android Keystore.</x:v>
-      </x:c>
-      <x:c r="E25" s="8" t="str"/>
-      <x:c r="F25" s="8" t="str"/>
-      <x:c r="G25" s="8" t="str"/>
-      <x:c r="H25" s="8" t="str"/>
-      <x:c r="I25" s="8" t="str"/>
-      <x:c r="J25" s="8" t="str"/>
-      <x:c r="K25" s="8" t="str"/>
-      <x:c r="L25" s="8" t="str"/>
+        <x:v>The operator enters and confirms the PIN inside MethodMesh. The form never stores the PIN, encryption key, random credential secret or encrypted envelope.</x:v>
+      </x:c>
+      <x:c r="E25" s="8"/>
+      <x:c r="F25" s="8"/>
+      <x:c r="G25" s="8"/>
+      <x:c r="H25" s="8"/>
+      <x:c r="I25" s="8"/>
+      <x:c r="J25" s="8"/>
+      <x:c r="K25" s="8"/>
+      <x:c r="L25" s="8"/>
+      <x:c r="M25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="8" t="str">
@@ -878,16 +903,17 @@
       <x:c r="B26" s="8" t="str">
         <x:v>credential_options_end</x:v>
       </x:c>
-      <x:c r="C26" s="8" t="str"/>
-      <x:c r="D26" s="8" t="str"/>
-      <x:c r="E26" s="8" t="str"/>
-      <x:c r="F26" s="8" t="str"/>
-      <x:c r="G26" s="8" t="str"/>
-      <x:c r="H26" s="8" t="str"/>
-      <x:c r="I26" s="8" t="str"/>
-      <x:c r="J26" s="8" t="str"/>
-      <x:c r="K26" s="8" t="str"/>
-      <x:c r="L26" s="8" t="str"/>
+      <x:c r="C26" s="8"/>
+      <x:c r="D26" s="8"/>
+      <x:c r="E26" s="8"/>
+      <x:c r="F26" s="8"/>
+      <x:c r="G26" s="8"/>
+      <x:c r="H26" s="8"/>
+      <x:c r="I26" s="8"/>
+      <x:c r="J26" s="8"/>
+      <x:c r="K26" s="8"/>
+      <x:c r="L26" s="8"/>
+      <x:c r="M26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="8" t="str">
@@ -900,20 +926,21 @@
         <x:v>Write and verify NFC credential</x:v>
       </x:c>
       <x:c r="D27" s="8" t="str">
-        <x:v>Complete provisioning in MethodMesh, then Commit to return here.</x:v>
-      </x:c>
-      <x:c r="E27" s="8" t="str"/>
-      <x:c r="F27" s="8" t="str"/>
-      <x:c r="G27" s="8" t="str"/>
-      <x:c r="H27" s="8" t="str"/>
-      <x:c r="I27" s="8" t="str"/>
+        <x:v>Tap the credential card, complete the MethodMesh provisioning workflow, then Commit to return here.</x:v>
+      </x:c>
+      <x:c r="E27" s="8"/>
+      <x:c r="F27" s="8"/>
+      <x:c r="G27" s="8"/>
+      <x:c r="H27" s="8"/>
+      <x:c r="I27" s="8"/>
       <x:c r="J27" s="8" t="str">
         <x:v>field-list</x:v>
       </x:c>
-      <x:c r="K27" s="8" t="str"/>
+      <x:c r="K27" s="8"/>
       <x:c r="L27" s="8" t="str">
         <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_overwrite_policy=${overwrite_policy_input},input_payload_mode='FULL',return_mode='flat')</x:v>
       </x:c>
+      <x:c r="M27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="8" t="str">
@@ -928,16 +955,17 @@
       <x:c r="D28" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E28" s="8" t="str"/>
-      <x:c r="F28" s="8" t="str"/>
-      <x:c r="G28" s="8" t="str"/>
-      <x:c r="H28" s="8" t="str"/>
-      <x:c r="I28" s="8" t="str"/>
+      <x:c r="E28" s="8"/>
+      <x:c r="F28" s="8"/>
+      <x:c r="G28" s="8"/>
+      <x:c r="H28" s="8"/>
+      <x:c r="I28" s="8"/>
       <x:c r="J28" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K28" s="8" t="str"/>
-      <x:c r="L28" s="8" t="str"/>
+      <x:c r="K28" s="8"/>
+      <x:c r="L28" s="8"/>
+      <x:c r="M28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="8" t="str">
@@ -952,16 +980,17 @@
       <x:c r="D29" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E29" s="8" t="str"/>
-      <x:c r="F29" s="8" t="str"/>
-      <x:c r="G29" s="8" t="str"/>
-      <x:c r="H29" s="8" t="str"/>
-      <x:c r="I29" s="8" t="str"/>
+      <x:c r="E29" s="8"/>
+      <x:c r="F29" s="8"/>
+      <x:c r="G29" s="8"/>
+      <x:c r="H29" s="8"/>
+      <x:c r="I29" s="8"/>
       <x:c r="J29" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K29" s="8" t="str"/>
-      <x:c r="L29" s="8" t="str"/>
+      <x:c r="K29" s="8"/>
+      <x:c r="L29" s="8"/>
+      <x:c r="M29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="8" t="str">
@@ -976,16 +1005,17 @@
       <x:c r="D30" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E30" s="8" t="str"/>
-      <x:c r="F30" s="8" t="str"/>
-      <x:c r="G30" s="8" t="str"/>
-      <x:c r="H30" s="8" t="str"/>
-      <x:c r="I30" s="8" t="str"/>
+      <x:c r="E30" s="8"/>
+      <x:c r="F30" s="8"/>
+      <x:c r="G30" s="8"/>
+      <x:c r="H30" s="8"/>
+      <x:c r="I30" s="8"/>
       <x:c r="J30" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K30" s="8" t="str"/>
-      <x:c r="L30" s="8" t="str"/>
+      <x:c r="K30" s="8"/>
+      <x:c r="L30" s="8"/>
+      <x:c r="M30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="8" t="str">
@@ -1000,16 +1030,17 @@
       <x:c r="D31" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E31" s="8" t="str"/>
-      <x:c r="F31" s="8" t="str"/>
-      <x:c r="G31" s="8" t="str"/>
-      <x:c r="H31" s="8" t="str"/>
-      <x:c r="I31" s="8" t="str"/>
+      <x:c r="E31" s="8"/>
+      <x:c r="F31" s="8"/>
+      <x:c r="G31" s="8"/>
+      <x:c r="H31" s="8"/>
+      <x:c r="I31" s="8"/>
       <x:c r="J31" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K31" s="8" t="str"/>
-      <x:c r="L31" s="8" t="str"/>
+      <x:c r="K31" s="8"/>
+      <x:c r="L31" s="8"/>
+      <x:c r="M31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="8" t="str">
@@ -1024,16 +1055,17 @@
       <x:c r="D32" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E32" s="8" t="str"/>
-      <x:c r="F32" s="8" t="str"/>
-      <x:c r="G32" s="8" t="str"/>
-      <x:c r="H32" s="8" t="str"/>
-      <x:c r="I32" s="8" t="str"/>
+      <x:c r="E32" s="8"/>
+      <x:c r="F32" s="8"/>
+      <x:c r="G32" s="8"/>
+      <x:c r="H32" s="8"/>
+      <x:c r="I32" s="8"/>
       <x:c r="J32" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K32" s="8" t="str"/>
-      <x:c r="L32" s="8" t="str"/>
+      <x:c r="K32" s="8"/>
+      <x:c r="L32" s="8"/>
+      <x:c r="M32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="8" t="str">
@@ -1048,16 +1080,17 @@
       <x:c r="D33" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E33" s="8" t="str"/>
-      <x:c r="F33" s="8" t="str"/>
-      <x:c r="G33" s="8" t="str"/>
-      <x:c r="H33" s="8" t="str"/>
-      <x:c r="I33" s="8" t="str"/>
+      <x:c r="E33" s="8"/>
+      <x:c r="F33" s="8"/>
+      <x:c r="G33" s="8"/>
+      <x:c r="H33" s="8"/>
+      <x:c r="I33" s="8"/>
       <x:c r="J33" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K33" s="8" t="str"/>
-      <x:c r="L33" s="8" t="str"/>
+      <x:c r="K33" s="8"/>
+      <x:c r="L33" s="8"/>
+      <x:c r="M33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="8" t="str">
@@ -1072,16 +1105,17 @@
       <x:c r="D34" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E34" s="8" t="str"/>
-      <x:c r="F34" s="8" t="str"/>
-      <x:c r="G34" s="8" t="str"/>
-      <x:c r="H34" s="8" t="str"/>
-      <x:c r="I34" s="8" t="str"/>
+      <x:c r="E34" s="8"/>
+      <x:c r="F34" s="8"/>
+      <x:c r="G34" s="8"/>
+      <x:c r="H34" s="8"/>
+      <x:c r="I34" s="8"/>
       <x:c r="J34" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K34" s="8" t="str"/>
-      <x:c r="L34" s="8" t="str"/>
+      <x:c r="K34" s="8"/>
+      <x:c r="L34" s="8"/>
+      <x:c r="M34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="8" t="str">
@@ -1096,16 +1130,17 @@
       <x:c r="D35" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E35" s="8" t="str"/>
-      <x:c r="F35" s="8" t="str"/>
-      <x:c r="G35" s="8" t="str"/>
-      <x:c r="H35" s="8" t="str"/>
-      <x:c r="I35" s="8" t="str"/>
+      <x:c r="E35" s="8"/>
+      <x:c r="F35" s="8"/>
+      <x:c r="G35" s="8"/>
+      <x:c r="H35" s="8"/>
+      <x:c r="I35" s="8"/>
       <x:c r="J35" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K35" s="8" t="str"/>
-      <x:c r="L35" s="8" t="str"/>
+      <x:c r="K35" s="8"/>
+      <x:c r="L35" s="8"/>
+      <x:c r="M35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="8" t="str">
@@ -1120,16 +1155,17 @@
       <x:c r="D36" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E36" s="8" t="str"/>
-      <x:c r="F36" s="8" t="str"/>
-      <x:c r="G36" s="8" t="str"/>
-      <x:c r="H36" s="8" t="str"/>
-      <x:c r="I36" s="8" t="str"/>
+      <x:c r="E36" s="8"/>
+      <x:c r="F36" s="8"/>
+      <x:c r="G36" s="8"/>
+      <x:c r="H36" s="8"/>
+      <x:c r="I36" s="8"/>
       <x:c r="J36" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K36" s="8" t="str"/>
-      <x:c r="L36" s="8" t="str"/>
+      <x:c r="K36" s="8"/>
+      <x:c r="L36" s="8"/>
+      <x:c r="M36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="8" t="str">
@@ -1144,16 +1180,17 @@
       <x:c r="D37" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E37" s="8" t="str"/>
-      <x:c r="F37" s="8" t="str"/>
-      <x:c r="G37" s="8" t="str"/>
-      <x:c r="H37" s="8" t="str"/>
-      <x:c r="I37" s="8" t="str"/>
+      <x:c r="E37" s="8"/>
+      <x:c r="F37" s="8"/>
+      <x:c r="G37" s="8"/>
+      <x:c r="H37" s="8"/>
+      <x:c r="I37" s="8"/>
       <x:c r="J37" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K37" s="8" t="str"/>
-      <x:c r="L37" s="8" t="str"/>
+      <x:c r="K37" s="8"/>
+      <x:c r="L37" s="8"/>
+      <x:c r="M37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="8" t="str">
@@ -1163,21 +1200,22 @@
         <x:v>issuer_key_id</x:v>
       </x:c>
       <x:c r="C38" s="8" t="str">
-        <x:v>Issuer short key ID</x:v>
+        <x:v>Issuer key ID</x:v>
       </x:c>
       <x:c r="D38" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E38" s="8" t="str"/>
-      <x:c r="F38" s="8" t="str"/>
-      <x:c r="G38" s="8" t="str"/>
-      <x:c r="H38" s="8" t="str"/>
-      <x:c r="I38" s="8" t="str"/>
+      <x:c r="E38" s="8"/>
+      <x:c r="F38" s="8"/>
+      <x:c r="G38" s="8"/>
+      <x:c r="H38" s="8"/>
+      <x:c r="I38" s="8"/>
       <x:c r="J38" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K38" s="8" t="str"/>
-      <x:c r="L38" s="8" t="str"/>
+      <x:c r="K38" s="8"/>
+      <x:c r="L38" s="8"/>
+      <x:c r="M38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="8" t="str">
@@ -1187,21 +1225,22 @@
         <x:v>issuer_public_key_fingerprint_sha256</x:v>
       </x:c>
       <x:c r="C39" s="8" t="str">
-        <x:v>Issuer public-key SHA-256 fingerprint</x:v>
+        <x:v>Issuer public key SHA-256 fingerprint</x:v>
       </x:c>
       <x:c r="D39" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
-      <x:c r="E39" s="8" t="str"/>
-      <x:c r="F39" s="8" t="str"/>
-      <x:c r="G39" s="8" t="str"/>
-      <x:c r="H39" s="8" t="str"/>
-      <x:c r="I39" s="8" t="str"/>
+        <x:v>Canonical full 64-character provisioning-device identity derived by MethodMesh from the issuer public key.</x:v>
+      </x:c>
+      <x:c r="E39" s="8"/>
+      <x:c r="F39" s="8"/>
+      <x:c r="G39" s="8"/>
+      <x:c r="H39" s="8"/>
+      <x:c r="I39" s="8"/>
       <x:c r="J39" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K39" s="8" t="str"/>
-      <x:c r="L39" s="8" t="str"/>
+      <x:c r="K39" s="8"/>
+      <x:c r="L39" s="8"/>
+      <x:c r="M39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="8" t="str">
@@ -1216,16 +1255,17 @@
       <x:c r="D40" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E40" s="8" t="str"/>
-      <x:c r="F40" s="8" t="str"/>
-      <x:c r="G40" s="8" t="str"/>
-      <x:c r="H40" s="8" t="str"/>
-      <x:c r="I40" s="8" t="str"/>
+      <x:c r="E40" s="8"/>
+      <x:c r="F40" s="8"/>
+      <x:c r="G40" s="8"/>
+      <x:c r="H40" s="8"/>
+      <x:c r="I40" s="8"/>
       <x:c r="J40" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K40" s="8" t="str"/>
-      <x:c r="L40" s="8" t="str"/>
+      <x:c r="K40" s="8"/>
+      <x:c r="L40" s="8"/>
+      <x:c r="M40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="8" t="str">
@@ -1240,16 +1280,17 @@
       <x:c r="D41" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E41" s="8" t="str"/>
-      <x:c r="F41" s="8" t="str"/>
-      <x:c r="G41" s="8" t="str"/>
-      <x:c r="H41" s="8" t="str"/>
-      <x:c r="I41" s="8" t="str"/>
+      <x:c r="E41" s="8"/>
+      <x:c r="F41" s="8"/>
+      <x:c r="G41" s="8"/>
+      <x:c r="H41" s="8"/>
+      <x:c r="I41" s="8"/>
       <x:c r="J41" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K41" s="8" t="str"/>
-      <x:c r="L41" s="8" t="str"/>
+      <x:c r="K41" s="8"/>
+      <x:c r="L41" s="8"/>
+      <x:c r="M41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="8" t="str">
@@ -1264,16 +1305,17 @@
       <x:c r="D42" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E42" s="8" t="str"/>
-      <x:c r="F42" s="8" t="str"/>
-      <x:c r="G42" s="8" t="str"/>
-      <x:c r="H42" s="8" t="str"/>
-      <x:c r="I42" s="8" t="str"/>
+      <x:c r="E42" s="8"/>
+      <x:c r="F42" s="8"/>
+      <x:c r="G42" s="8"/>
+      <x:c r="H42" s="8"/>
+      <x:c r="I42" s="8"/>
       <x:c r="J42" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K42" s="8" t="str"/>
-      <x:c r="L42" s="8" t="str"/>
+      <x:c r="K42" s="8"/>
+      <x:c r="L42" s="8"/>
+      <x:c r="M42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="8" t="str">
@@ -1288,16 +1330,17 @@
       <x:c r="D43" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E43" s="8" t="str"/>
-      <x:c r="F43" s="8" t="str"/>
-      <x:c r="G43" s="8" t="str"/>
-      <x:c r="H43" s="8" t="str"/>
-      <x:c r="I43" s="8" t="str"/>
+      <x:c r="E43" s="8"/>
+      <x:c r="F43" s="8"/>
+      <x:c r="G43" s="8"/>
+      <x:c r="H43" s="8"/>
+      <x:c r="I43" s="8"/>
       <x:c r="J43" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K43" s="8" t="str"/>
-      <x:c r="L43" s="8" t="str"/>
+      <x:c r="K43" s="8"/>
+      <x:c r="L43" s="8"/>
+      <x:c r="M43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="8" t="str">
@@ -1312,16 +1355,17 @@
       <x:c r="D44" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E44" s="8" t="str"/>
-      <x:c r="F44" s="8" t="str"/>
-      <x:c r="G44" s="8" t="str"/>
-      <x:c r="H44" s="8" t="str"/>
-      <x:c r="I44" s="8" t="str"/>
+      <x:c r="E44" s="8"/>
+      <x:c r="F44" s="8"/>
+      <x:c r="G44" s="8"/>
+      <x:c r="H44" s="8"/>
+      <x:c r="I44" s="8"/>
       <x:c r="J44" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K44" s="8" t="str"/>
-      <x:c r="L44" s="8" t="str"/>
+      <x:c r="K44" s="8"/>
+      <x:c r="L44" s="8"/>
+      <x:c r="M44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="8" t="str">
@@ -1336,16 +1380,17 @@
       <x:c r="D45" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E45" s="8" t="str"/>
-      <x:c r="F45" s="8" t="str"/>
-      <x:c r="G45" s="8" t="str"/>
-      <x:c r="H45" s="8" t="str"/>
-      <x:c r="I45" s="8" t="str"/>
+      <x:c r="E45" s="8"/>
+      <x:c r="F45" s="8"/>
+      <x:c r="G45" s="8"/>
+      <x:c r="H45" s="8"/>
+      <x:c r="I45" s="8"/>
       <x:c r="J45" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K45" s="8" t="str"/>
-      <x:c r="L45" s="8" t="str"/>
+      <x:c r="K45" s="8"/>
+      <x:c r="L45" s="8"/>
+      <x:c r="M45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="8" t="str">
@@ -1360,16 +1405,17 @@
       <x:c r="D46" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E46" s="8" t="str"/>
-      <x:c r="F46" s="8" t="str"/>
-      <x:c r="G46" s="8" t="str"/>
-      <x:c r="H46" s="8" t="str"/>
-      <x:c r="I46" s="8" t="str"/>
+      <x:c r="E46" s="8"/>
+      <x:c r="F46" s="8"/>
+      <x:c r="G46" s="8"/>
+      <x:c r="H46" s="8"/>
+      <x:c r="I46" s="8"/>
       <x:c r="J46" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K46" s="8" t="str"/>
-      <x:c r="L46" s="8" t="str"/>
+      <x:c r="K46" s="8"/>
+      <x:c r="L46" s="8"/>
+      <x:c r="M46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="8" t="str">
@@ -1384,16 +1430,17 @@
       <x:c r="D47" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E47" s="8" t="str"/>
-      <x:c r="F47" s="8" t="str"/>
-      <x:c r="G47" s="8" t="str"/>
-      <x:c r="H47" s="8" t="str"/>
-      <x:c r="I47" s="8" t="str"/>
+      <x:c r="E47" s="8"/>
+      <x:c r="F47" s="8"/>
+      <x:c r="G47" s="8"/>
+      <x:c r="H47" s="8"/>
+      <x:c r="I47" s="8"/>
       <x:c r="J47" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K47" s="8" t="str"/>
-      <x:c r="L47" s="8" t="str"/>
+      <x:c r="K47" s="8"/>
+      <x:c r="L47" s="8"/>
+      <x:c r="M47"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="8" t="str">
@@ -1408,16 +1455,17 @@
       <x:c r="D48" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E48" s="8" t="str"/>
-      <x:c r="F48" s="8" t="str"/>
-      <x:c r="G48" s="8" t="str"/>
-      <x:c r="H48" s="8" t="str"/>
-      <x:c r="I48" s="8" t="str"/>
+      <x:c r="E48" s="8"/>
+      <x:c r="F48" s="8"/>
+      <x:c r="G48" s="8"/>
+      <x:c r="H48" s="8"/>
+      <x:c r="I48" s="8"/>
       <x:c r="J48" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K48" s="8" t="str"/>
-      <x:c r="L48" s="8" t="str"/>
+      <x:c r="K48" s="8"/>
+      <x:c r="L48" s="8"/>
+      <x:c r="M48"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="8" t="str">
@@ -1432,16 +1480,17 @@
       <x:c r="D49" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E49" s="8" t="str"/>
-      <x:c r="F49" s="8" t="str"/>
-      <x:c r="G49" s="8" t="str"/>
-      <x:c r="H49" s="8" t="str"/>
-      <x:c r="I49" s="8" t="str"/>
+      <x:c r="E49" s="8"/>
+      <x:c r="F49" s="8"/>
+      <x:c r="G49" s="8"/>
+      <x:c r="H49" s="8"/>
+      <x:c r="I49" s="8"/>
       <x:c r="J49" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K49" s="8" t="str"/>
-      <x:c r="L49" s="8" t="str"/>
+      <x:c r="K49" s="8"/>
+      <x:c r="L49" s="8"/>
+      <x:c r="M49"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="8" t="str">
@@ -1456,16 +1505,17 @@
       <x:c r="D50" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E50" s="8" t="str"/>
-      <x:c r="F50" s="8" t="str"/>
-      <x:c r="G50" s="8" t="str"/>
-      <x:c r="H50" s="8" t="str"/>
-      <x:c r="I50" s="8" t="str"/>
+      <x:c r="E50" s="8"/>
+      <x:c r="F50" s="8"/>
+      <x:c r="G50" s="8"/>
+      <x:c r="H50" s="8"/>
+      <x:c r="I50" s="8"/>
       <x:c r="J50" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K50" s="8" t="str"/>
-      <x:c r="L50" s="8" t="str"/>
+      <x:c r="K50" s="8"/>
+      <x:c r="L50" s="8"/>
+      <x:c r="M50"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="8" t="str">
@@ -1480,16 +1530,17 @@
       <x:c r="D51" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E51" s="8" t="str"/>
-      <x:c r="F51" s="8" t="str"/>
-      <x:c r="G51" s="8" t="str"/>
-      <x:c r="H51" s="8" t="str"/>
-      <x:c r="I51" s="8" t="str"/>
+      <x:c r="E51" s="8"/>
+      <x:c r="F51" s="8"/>
+      <x:c r="G51" s="8"/>
+      <x:c r="H51" s="8"/>
+      <x:c r="I51" s="8"/>
       <x:c r="J51" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K51" s="8" t="str"/>
-      <x:c r="L51" s="8" t="str"/>
+      <x:c r="K51" s="8"/>
+      <x:c r="L51" s="8"/>
+      <x:c r="M51"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="8" t="str">
@@ -1504,16 +1555,17 @@
       <x:c r="D52" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E52" s="8" t="str"/>
-      <x:c r="F52" s="8" t="str"/>
-      <x:c r="G52" s="8" t="str"/>
-      <x:c r="H52" s="8" t="str"/>
-      <x:c r="I52" s="8" t="str"/>
+      <x:c r="E52" s="8"/>
+      <x:c r="F52" s="8"/>
+      <x:c r="G52" s="8"/>
+      <x:c r="H52" s="8"/>
+      <x:c r="I52" s="8"/>
       <x:c r="J52" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K52" s="8" t="str"/>
-      <x:c r="L52" s="8" t="str"/>
+      <x:c r="K52" s="8"/>
+      <x:c r="L52" s="8"/>
+      <x:c r="M52"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="8" t="str">
@@ -1528,16 +1580,17 @@
       <x:c r="D53" s="8" t="str">
         <x:v>Returned by MethodMesh.</x:v>
       </x:c>
-      <x:c r="E53" s="8" t="str"/>
-      <x:c r="F53" s="8" t="str"/>
-      <x:c r="G53" s="8" t="str"/>
-      <x:c r="H53" s="8" t="str"/>
-      <x:c r="I53" s="8" t="str"/>
+      <x:c r="E53" s="8"/>
+      <x:c r="F53" s="8"/>
+      <x:c r="G53" s="8"/>
+      <x:c r="H53" s="8"/>
+      <x:c r="I53" s="8"/>
       <x:c r="J53" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="K53" s="8" t="str"/>
-      <x:c r="L53" s="8" t="str"/>
+      <x:c r="K53" s="8"/>
+      <x:c r="L53" s="8"/>
+      <x:c r="M53"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="8" t="str">
@@ -1546,16 +1599,17 @@
       <x:c r="B54" s="8" t="str">
         <x:v>run_nfc_credential_provisioning_end</x:v>
       </x:c>
-      <x:c r="C54" s="8" t="str"/>
-      <x:c r="D54" s="8" t="str"/>
-      <x:c r="E54" s="8" t="str"/>
-      <x:c r="F54" s="8" t="str"/>
-      <x:c r="G54" s="8" t="str"/>
-      <x:c r="H54" s="8" t="str"/>
-      <x:c r="I54" s="8" t="str"/>
-      <x:c r="J54" s="8" t="str"/>
-      <x:c r="K54" s="8" t="str"/>
-      <x:c r="L54" s="8" t="str"/>
+      <x:c r="C54" s="8"/>
+      <x:c r="D54" s="8"/>
+      <x:c r="E54" s="8"/>
+      <x:c r="F54" s="8"/>
+      <x:c r="G54" s="8"/>
+      <x:c r="H54" s="8"/>
+      <x:c r="I54" s="8"/>
+      <x:c r="J54" s="8"/>
+      <x:c r="K54" s="8"/>
+      <x:c r="L54" s="8"/>
+      <x:c r="M54"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="8" t="str">
@@ -1568,18 +1622,19 @@
         <x:v>Credential provisioning result</x:v>
       </x:c>
       <x:c r="D55" s="8" t="str">
-        <x:v>Credential ${credential_id}; write verified ${write_verified}; issuer ${issuer_key_id}; fingerprint ${issuer_public_key_fingerprint_sha256}.</x:v>
-      </x:c>
-      <x:c r="E55" s="8" t="str"/>
+        <x:v>Credential ${credential_id}; MethodMesh status ${methodmesh_status}; write verified ${write_verified}; issuer ${issuer_key_id}; issuer fingerprint ${issuer_public_key_fingerprint_sha256}.</x:v>
+      </x:c>
+      <x:c r="E55" s="8"/>
       <x:c r="F55" s="8" t="str">
         <x:v>${methodmesh_status} != ''</x:v>
       </x:c>
-      <x:c r="G55" s="8" t="str"/>
-      <x:c r="H55" s="8" t="str"/>
-      <x:c r="I55" s="8" t="str"/>
-      <x:c r="J55" s="8" t="str"/>
-      <x:c r="K55" s="8" t="str"/>
-      <x:c r="L55" s="8" t="str"/>
+      <x:c r="G55" s="8"/>
+      <x:c r="H55" s="8"/>
+      <x:c r="I55" s="8"/>
+      <x:c r="J55" s="8"/>
+      <x:c r="K55" s="8"/>
+      <x:c r="L55" s="8"/>
+      <x:c r="M55"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="8" t="str">
@@ -1592,16 +1647,17 @@
         <x:v>Registry record retained</x:v>
       </x:c>
       <x:c r="D56" s="8" t="str">
-        <x:v>Name, role, site and administrative validity remain in ODK. The returned full issuer fingerprint is the value to place in the study's offline trusted-issuer configuration.</x:v>
-      </x:c>
-      <x:c r="E56" s="8" t="str"/>
-      <x:c r="F56" s="8" t="str"/>
-      <x:c r="G56" s="8" t="str"/>
-      <x:c r="H56" s="8" t="str"/>
-      <x:c r="I56" s="8" t="str"/>
-      <x:c r="J56" s="8" t="str"/>
-      <x:c r="K56" s="8" t="str"/>
-      <x:c r="L56" s="8" t="str"/>
+        <x:v>Name, role, site, start/end dates, authorisation and issuance reason remain in the study credential registry and are linked to credential_id. The full issuer_public_key_fingerprint_sha256 is the canonical provisioning-device identity used later for central reconciliation. These governance fields are not silently added to the ROSC1 card.</x:v>
+      </x:c>
+      <x:c r="E56" s="8"/>
+      <x:c r="F56" s="8"/>
+      <x:c r="G56" s="8"/>
+      <x:c r="H56" s="8"/>
+      <x:c r="I56" s="8"/>
+      <x:c r="J56" s="8"/>
+      <x:c r="K56" s="8"/>
+      <x:c r="L56" s="8"/>
+      <x:c r="M56"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="8"/>
@@ -1616,6 +1672,7 @@
       <x:c r="J57" s="8"/>
       <x:c r="K57" s="8"/>
       <x:c r="L57" s="8"/>
+      <x:c r="M57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="8"/>
@@ -1630,6 +1687,7 @@
       <x:c r="J58" s="8"/>
       <x:c r="K58" s="8"/>
       <x:c r="L58" s="8"/>
+      <x:c r="M58"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="8"/>
@@ -1644,6 +1702,7 @@
       <x:c r="J59" s="8"/>
       <x:c r="K59" s="8"/>
       <x:c r="L59" s="8"/>
+      <x:c r="M59"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="8"/>
@@ -1658,6 +1717,7 @@
       <x:c r="J60" s="8"/>
       <x:c r="K60" s="8"/>
       <x:c r="L60" s="8"/>
+      <x:c r="M60"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="8"/>
@@ -1672,6 +1732,7 @@
       <x:c r="J61" s="8"/>
       <x:c r="K61" s="8"/>
       <x:c r="L61" s="8"/>
+      <x:c r="M61"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="8"/>
@@ -1686,6 +1747,7 @@
       <x:c r="J62" s="8"/>
       <x:c r="K62" s="8"/>
       <x:c r="L62" s="8"/>
+      <x:c r="M62"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="8"/>
@@ -1700,6 +1762,7 @@
       <x:c r="J63" s="8"/>
       <x:c r="K63" s="8"/>
       <x:c r="L63" s="8"/>
+      <x:c r="M63"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="8"/>
@@ -1714,6 +1777,7 @@
       <x:c r="J64" s="8"/>
       <x:c r="K64" s="8"/>
       <x:c r="L64" s="8"/>
+      <x:c r="M64"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="8"/>
@@ -1728,6 +1792,7 @@
       <x:c r="J65" s="8"/>
       <x:c r="K65" s="8"/>
       <x:c r="L65" s="8"/>
+      <x:c r="M65"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="8"/>
@@ -1742,6 +1807,7 @@
       <x:c r="J66" s="8"/>
       <x:c r="K66" s="8"/>
       <x:c r="L66" s="8"/>
+      <x:c r="M66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="8"/>
@@ -1756,6 +1822,7 @@
       <x:c r="J67" s="8"/>
       <x:c r="K67" s="8"/>
       <x:c r="L67" s="8"/>
+      <x:c r="M67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="8"/>
@@ -1770,6 +1837,7 @@
       <x:c r="J68" s="8"/>
       <x:c r="K68" s="8"/>
       <x:c r="L68" s="8"/>
+      <x:c r="M68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="8"/>
@@ -1784,6 +1852,7 @@
       <x:c r="J69" s="8"/>
       <x:c r="K69" s="8"/>
       <x:c r="L69" s="8"/>
+      <x:c r="M69"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="8"/>
@@ -1798,6 +1867,7 @@
       <x:c r="J70" s="8"/>
       <x:c r="K70" s="8"/>
       <x:c r="L70" s="8"/>
+      <x:c r="M70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="8"/>
@@ -1812,6 +1882,7 @@
       <x:c r="J71" s="8"/>
       <x:c r="K71" s="8"/>
       <x:c r="L71" s="8"/>
+      <x:c r="M71"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="8"/>
@@ -1826,6 +1897,7 @@
       <x:c r="J72" s="8"/>
       <x:c r="K72" s="8"/>
       <x:c r="L72" s="8"/>
+      <x:c r="M72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="8"/>
@@ -1840,6 +1912,7 @@
       <x:c r="J73" s="8"/>
       <x:c r="K73" s="8"/>
       <x:c r="L73" s="8"/>
+      <x:c r="M73"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="8"/>
@@ -1854,6 +1927,7 @@
       <x:c r="J74" s="8"/>
       <x:c r="K74" s="8"/>
       <x:c r="L74" s="8"/>
+      <x:c r="M74"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="8"/>
@@ -1868,6 +1942,7 @@
       <x:c r="J75" s="8"/>
       <x:c r="K75" s="8"/>
       <x:c r="L75" s="8"/>
+      <x:c r="M75"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="8"/>
@@ -1882,6 +1957,7 @@
       <x:c r="J76" s="8"/>
       <x:c r="K76" s="8"/>
       <x:c r="L76" s="8"/>
+      <x:c r="M76"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="8"/>
@@ -1896,6 +1972,7 @@
       <x:c r="J77" s="8"/>
       <x:c r="K77" s="8"/>
       <x:c r="L77" s="8"/>
+      <x:c r="M77"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="8"/>
@@ -1910,6 +1987,7 @@
       <x:c r="J78" s="8"/>
       <x:c r="K78" s="8"/>
       <x:c r="L78" s="8"/>
+      <x:c r="M78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="8"/>
@@ -1924,6 +2002,7 @@
       <x:c r="J79" s="8"/>
       <x:c r="K79" s="8"/>
       <x:c r="L79" s="8"/>
+      <x:c r="M79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="8"/>
@@ -1938,6 +2017,7 @@
       <x:c r="J80" s="8"/>
       <x:c r="K80" s="8"/>
       <x:c r="L80" s="8"/>
+      <x:c r="M80"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="8"/>
@@ -3059,6 +3139,566 @@
       <x:c r="K160" s="8"/>
       <x:c r="L160" s="8"/>
     </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="8"/>
+      <x:c r="B161" s="8"/>
+      <x:c r="C161" s="8"/>
+      <x:c r="D161" s="8"/>
+      <x:c r="E161" s="8"/>
+      <x:c r="F161" s="8"/>
+      <x:c r="G161" s="8"/>
+      <x:c r="H161" s="8"/>
+      <x:c r="I161" s="8"/>
+      <x:c r="J161" s="8"/>
+      <x:c r="K161" s="8"/>
+      <x:c r="L161" s="8"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="8"/>
+      <x:c r="B162" s="8"/>
+      <x:c r="C162" s="8"/>
+      <x:c r="D162" s="8"/>
+      <x:c r="E162" s="8"/>
+      <x:c r="F162" s="8"/>
+      <x:c r="G162" s="8"/>
+      <x:c r="H162" s="8"/>
+      <x:c r="I162" s="8"/>
+      <x:c r="J162" s="8"/>
+      <x:c r="K162" s="8"/>
+      <x:c r="L162" s="8"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="8"/>
+      <x:c r="B163" s="8"/>
+      <x:c r="C163" s="8"/>
+      <x:c r="D163" s="8"/>
+      <x:c r="E163" s="8"/>
+      <x:c r="F163" s="8"/>
+      <x:c r="G163" s="8"/>
+      <x:c r="H163" s="8"/>
+      <x:c r="I163" s="8"/>
+      <x:c r="J163" s="8"/>
+      <x:c r="K163" s="8"/>
+      <x:c r="L163" s="8"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="8"/>
+      <x:c r="B164" s="8"/>
+      <x:c r="C164" s="8"/>
+      <x:c r="D164" s="8"/>
+      <x:c r="E164" s="8"/>
+      <x:c r="F164" s="8"/>
+      <x:c r="G164" s="8"/>
+      <x:c r="H164" s="8"/>
+      <x:c r="I164" s="8"/>
+      <x:c r="J164" s="8"/>
+      <x:c r="K164" s="8"/>
+      <x:c r="L164" s="8"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="8"/>
+      <x:c r="B165" s="8"/>
+      <x:c r="C165" s="8"/>
+      <x:c r="D165" s="8"/>
+      <x:c r="E165" s="8"/>
+      <x:c r="F165" s="8"/>
+      <x:c r="G165" s="8"/>
+      <x:c r="H165" s="8"/>
+      <x:c r="I165" s="8"/>
+      <x:c r="J165" s="8"/>
+      <x:c r="K165" s="8"/>
+      <x:c r="L165" s="8"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="8"/>
+      <x:c r="B166" s="8"/>
+      <x:c r="C166" s="8"/>
+      <x:c r="D166" s="8"/>
+      <x:c r="E166" s="8"/>
+      <x:c r="F166" s="8"/>
+      <x:c r="G166" s="8"/>
+      <x:c r="H166" s="8"/>
+      <x:c r="I166" s="8"/>
+      <x:c r="J166" s="8"/>
+      <x:c r="K166" s="8"/>
+      <x:c r="L166" s="8"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="8"/>
+      <x:c r="B167" s="8"/>
+      <x:c r="C167" s="8"/>
+      <x:c r="D167" s="8"/>
+      <x:c r="E167" s="8"/>
+      <x:c r="F167" s="8"/>
+      <x:c r="G167" s="8"/>
+      <x:c r="H167" s="8"/>
+      <x:c r="I167" s="8"/>
+      <x:c r="J167" s="8"/>
+      <x:c r="K167" s="8"/>
+      <x:c r="L167" s="8"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="8"/>
+      <x:c r="B168" s="8"/>
+      <x:c r="C168" s="8"/>
+      <x:c r="D168" s="8"/>
+      <x:c r="E168" s="8"/>
+      <x:c r="F168" s="8"/>
+      <x:c r="G168" s="8"/>
+      <x:c r="H168" s="8"/>
+      <x:c r="I168" s="8"/>
+      <x:c r="J168" s="8"/>
+      <x:c r="K168" s="8"/>
+      <x:c r="L168" s="8"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="8"/>
+      <x:c r="B169" s="8"/>
+      <x:c r="C169" s="8"/>
+      <x:c r="D169" s="8"/>
+      <x:c r="E169" s="8"/>
+      <x:c r="F169" s="8"/>
+      <x:c r="G169" s="8"/>
+      <x:c r="H169" s="8"/>
+      <x:c r="I169" s="8"/>
+      <x:c r="J169" s="8"/>
+      <x:c r="K169" s="8"/>
+      <x:c r="L169" s="8"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="8"/>
+      <x:c r="B170" s="8"/>
+      <x:c r="C170" s="8"/>
+      <x:c r="D170" s="8"/>
+      <x:c r="E170" s="8"/>
+      <x:c r="F170" s="8"/>
+      <x:c r="G170" s="8"/>
+      <x:c r="H170" s="8"/>
+      <x:c r="I170" s="8"/>
+      <x:c r="J170" s="8"/>
+      <x:c r="K170" s="8"/>
+      <x:c r="L170" s="8"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="8"/>
+      <x:c r="B171" s="8"/>
+      <x:c r="C171" s="8"/>
+      <x:c r="D171" s="8"/>
+      <x:c r="E171" s="8"/>
+      <x:c r="F171" s="8"/>
+      <x:c r="G171" s="8"/>
+      <x:c r="H171" s="8"/>
+      <x:c r="I171" s="8"/>
+      <x:c r="J171" s="8"/>
+      <x:c r="K171" s="8"/>
+      <x:c r="L171" s="8"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="8"/>
+      <x:c r="B172" s="8"/>
+      <x:c r="C172" s="8"/>
+      <x:c r="D172" s="8"/>
+      <x:c r="E172" s="8"/>
+      <x:c r="F172" s="8"/>
+      <x:c r="G172" s="8"/>
+      <x:c r="H172" s="8"/>
+      <x:c r="I172" s="8"/>
+      <x:c r="J172" s="8"/>
+      <x:c r="K172" s="8"/>
+      <x:c r="L172" s="8"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="8"/>
+      <x:c r="B173" s="8"/>
+      <x:c r="C173" s="8"/>
+      <x:c r="D173" s="8"/>
+      <x:c r="E173" s="8"/>
+      <x:c r="F173" s="8"/>
+      <x:c r="G173" s="8"/>
+      <x:c r="H173" s="8"/>
+      <x:c r="I173" s="8"/>
+      <x:c r="J173" s="8"/>
+      <x:c r="K173" s="8"/>
+      <x:c r="L173" s="8"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="8"/>
+      <x:c r="B174" s="8"/>
+      <x:c r="C174" s="8"/>
+      <x:c r="D174" s="8"/>
+      <x:c r="E174" s="8"/>
+      <x:c r="F174" s="8"/>
+      <x:c r="G174" s="8"/>
+      <x:c r="H174" s="8"/>
+      <x:c r="I174" s="8"/>
+      <x:c r="J174" s="8"/>
+      <x:c r="K174" s="8"/>
+      <x:c r="L174" s="8"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="8"/>
+      <x:c r="B175" s="8"/>
+      <x:c r="C175" s="8"/>
+      <x:c r="D175" s="8"/>
+      <x:c r="E175" s="8"/>
+      <x:c r="F175" s="8"/>
+      <x:c r="G175" s="8"/>
+      <x:c r="H175" s="8"/>
+      <x:c r="I175" s="8"/>
+      <x:c r="J175" s="8"/>
+      <x:c r="K175" s="8"/>
+      <x:c r="L175" s="8"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="8"/>
+      <x:c r="B176" s="8"/>
+      <x:c r="C176" s="8"/>
+      <x:c r="D176" s="8"/>
+      <x:c r="E176" s="8"/>
+      <x:c r="F176" s="8"/>
+      <x:c r="G176" s="8"/>
+      <x:c r="H176" s="8"/>
+      <x:c r="I176" s="8"/>
+      <x:c r="J176" s="8"/>
+      <x:c r="K176" s="8"/>
+      <x:c r="L176" s="8"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="8"/>
+      <x:c r="B177" s="8"/>
+      <x:c r="C177" s="8"/>
+      <x:c r="D177" s="8"/>
+      <x:c r="E177" s="8"/>
+      <x:c r="F177" s="8"/>
+      <x:c r="G177" s="8"/>
+      <x:c r="H177" s="8"/>
+      <x:c r="I177" s="8"/>
+      <x:c r="J177" s="8"/>
+      <x:c r="K177" s="8"/>
+      <x:c r="L177" s="8"/>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="8"/>
+      <x:c r="B178" s="8"/>
+      <x:c r="C178" s="8"/>
+      <x:c r="D178" s="8"/>
+      <x:c r="E178" s="8"/>
+      <x:c r="F178" s="8"/>
+      <x:c r="G178" s="8"/>
+      <x:c r="H178" s="8"/>
+      <x:c r="I178" s="8"/>
+      <x:c r="J178" s="8"/>
+      <x:c r="K178" s="8"/>
+      <x:c r="L178" s="8"/>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="8"/>
+      <x:c r="B179" s="8"/>
+      <x:c r="C179" s="8"/>
+      <x:c r="D179" s="8"/>
+      <x:c r="E179" s="8"/>
+      <x:c r="F179" s="8"/>
+      <x:c r="G179" s="8"/>
+      <x:c r="H179" s="8"/>
+      <x:c r="I179" s="8"/>
+      <x:c r="J179" s="8"/>
+      <x:c r="K179" s="8"/>
+      <x:c r="L179" s="8"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="8"/>
+      <x:c r="B180" s="8"/>
+      <x:c r="C180" s="8"/>
+      <x:c r="D180" s="8"/>
+      <x:c r="E180" s="8"/>
+      <x:c r="F180" s="8"/>
+      <x:c r="G180" s="8"/>
+      <x:c r="H180" s="8"/>
+      <x:c r="I180" s="8"/>
+      <x:c r="J180" s="8"/>
+      <x:c r="K180" s="8"/>
+      <x:c r="L180" s="8"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="8"/>
+      <x:c r="B181" s="8"/>
+      <x:c r="C181" s="8"/>
+      <x:c r="D181" s="8"/>
+      <x:c r="E181" s="8"/>
+      <x:c r="F181" s="8"/>
+      <x:c r="G181" s="8"/>
+      <x:c r="H181" s="8"/>
+      <x:c r="I181" s="8"/>
+      <x:c r="J181" s="8"/>
+      <x:c r="K181" s="8"/>
+      <x:c r="L181" s="8"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="8"/>
+      <x:c r="B182" s="8"/>
+      <x:c r="C182" s="8"/>
+      <x:c r="D182" s="8"/>
+      <x:c r="E182" s="8"/>
+      <x:c r="F182" s="8"/>
+      <x:c r="G182" s="8"/>
+      <x:c r="H182" s="8"/>
+      <x:c r="I182" s="8"/>
+      <x:c r="J182" s="8"/>
+      <x:c r="K182" s="8"/>
+      <x:c r="L182" s="8"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="8"/>
+      <x:c r="B183" s="8"/>
+      <x:c r="C183" s="8"/>
+      <x:c r="D183" s="8"/>
+      <x:c r="E183" s="8"/>
+      <x:c r="F183" s="8"/>
+      <x:c r="G183" s="8"/>
+      <x:c r="H183" s="8"/>
+      <x:c r="I183" s="8"/>
+      <x:c r="J183" s="8"/>
+      <x:c r="K183" s="8"/>
+      <x:c r="L183" s="8"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="8"/>
+      <x:c r="B184" s="8"/>
+      <x:c r="C184" s="8"/>
+      <x:c r="D184" s="8"/>
+      <x:c r="E184" s="8"/>
+      <x:c r="F184" s="8"/>
+      <x:c r="G184" s="8"/>
+      <x:c r="H184" s="8"/>
+      <x:c r="I184" s="8"/>
+      <x:c r="J184" s="8"/>
+      <x:c r="K184" s="8"/>
+      <x:c r="L184" s="8"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" s="8"/>
+      <x:c r="B185" s="8"/>
+      <x:c r="C185" s="8"/>
+      <x:c r="D185" s="8"/>
+      <x:c r="E185" s="8"/>
+      <x:c r="F185" s="8"/>
+      <x:c r="G185" s="8"/>
+      <x:c r="H185" s="8"/>
+      <x:c r="I185" s="8"/>
+      <x:c r="J185" s="8"/>
+      <x:c r="K185" s="8"/>
+      <x:c r="L185" s="8"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" s="8"/>
+      <x:c r="B186" s="8"/>
+      <x:c r="C186" s="8"/>
+      <x:c r="D186" s="8"/>
+      <x:c r="E186" s="8"/>
+      <x:c r="F186" s="8"/>
+      <x:c r="G186" s="8"/>
+      <x:c r="H186" s="8"/>
+      <x:c r="I186" s="8"/>
+      <x:c r="J186" s="8"/>
+      <x:c r="K186" s="8"/>
+      <x:c r="L186" s="8"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" s="8"/>
+      <x:c r="B187" s="8"/>
+      <x:c r="C187" s="8"/>
+      <x:c r="D187" s="8"/>
+      <x:c r="E187" s="8"/>
+      <x:c r="F187" s="8"/>
+      <x:c r="G187" s="8"/>
+      <x:c r="H187" s="8"/>
+      <x:c r="I187" s="8"/>
+      <x:c r="J187" s="8"/>
+      <x:c r="K187" s="8"/>
+      <x:c r="L187" s="8"/>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" s="8"/>
+      <x:c r="B188" s="8"/>
+      <x:c r="C188" s="8"/>
+      <x:c r="D188" s="8"/>
+      <x:c r="E188" s="8"/>
+      <x:c r="F188" s="8"/>
+      <x:c r="G188" s="8"/>
+      <x:c r="H188" s="8"/>
+      <x:c r="I188" s="8"/>
+      <x:c r="J188" s="8"/>
+      <x:c r="K188" s="8"/>
+      <x:c r="L188" s="8"/>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" s="8"/>
+      <x:c r="B189" s="8"/>
+      <x:c r="C189" s="8"/>
+      <x:c r="D189" s="8"/>
+      <x:c r="E189" s="8"/>
+      <x:c r="F189" s="8"/>
+      <x:c r="G189" s="8"/>
+      <x:c r="H189" s="8"/>
+      <x:c r="I189" s="8"/>
+      <x:c r="J189" s="8"/>
+      <x:c r="K189" s="8"/>
+      <x:c r="L189" s="8"/>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" s="8"/>
+      <x:c r="B190" s="8"/>
+      <x:c r="C190" s="8"/>
+      <x:c r="D190" s="8"/>
+      <x:c r="E190" s="8"/>
+      <x:c r="F190" s="8"/>
+      <x:c r="G190" s="8"/>
+      <x:c r="H190" s="8"/>
+      <x:c r="I190" s="8"/>
+      <x:c r="J190" s="8"/>
+      <x:c r="K190" s="8"/>
+      <x:c r="L190" s="8"/>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" s="8"/>
+      <x:c r="B191" s="8"/>
+      <x:c r="C191" s="8"/>
+      <x:c r="D191" s="8"/>
+      <x:c r="E191" s="8"/>
+      <x:c r="F191" s="8"/>
+      <x:c r="G191" s="8"/>
+      <x:c r="H191" s="8"/>
+      <x:c r="I191" s="8"/>
+      <x:c r="J191" s="8"/>
+      <x:c r="K191" s="8"/>
+      <x:c r="L191" s="8"/>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" s="8"/>
+      <x:c r="B192" s="8"/>
+      <x:c r="C192" s="8"/>
+      <x:c r="D192" s="8"/>
+      <x:c r="E192" s="8"/>
+      <x:c r="F192" s="8"/>
+      <x:c r="G192" s="8"/>
+      <x:c r="H192" s="8"/>
+      <x:c r="I192" s="8"/>
+      <x:c r="J192" s="8"/>
+      <x:c r="K192" s="8"/>
+      <x:c r="L192" s="8"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="8"/>
+      <x:c r="B193" s="8"/>
+      <x:c r="C193" s="8"/>
+      <x:c r="D193" s="8"/>
+      <x:c r="E193" s="8"/>
+      <x:c r="F193" s="8"/>
+      <x:c r="G193" s="8"/>
+      <x:c r="H193" s="8"/>
+      <x:c r="I193" s="8"/>
+      <x:c r="J193" s="8"/>
+      <x:c r="K193" s="8"/>
+      <x:c r="L193" s="8"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" s="8"/>
+      <x:c r="B194" s="8"/>
+      <x:c r="C194" s="8"/>
+      <x:c r="D194" s="8"/>
+      <x:c r="E194" s="8"/>
+      <x:c r="F194" s="8"/>
+      <x:c r="G194" s="8"/>
+      <x:c r="H194" s="8"/>
+      <x:c r="I194" s="8"/>
+      <x:c r="J194" s="8"/>
+      <x:c r="K194" s="8"/>
+      <x:c r="L194" s="8"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="8"/>
+      <x:c r="B195" s="8"/>
+      <x:c r="C195" s="8"/>
+      <x:c r="D195" s="8"/>
+      <x:c r="E195" s="8"/>
+      <x:c r="F195" s="8"/>
+      <x:c r="G195" s="8"/>
+      <x:c r="H195" s="8"/>
+      <x:c r="I195" s="8"/>
+      <x:c r="J195" s="8"/>
+      <x:c r="K195" s="8"/>
+      <x:c r="L195" s="8"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="8"/>
+      <x:c r="B196" s="8"/>
+      <x:c r="C196" s="8"/>
+      <x:c r="D196" s="8"/>
+      <x:c r="E196" s="8"/>
+      <x:c r="F196" s="8"/>
+      <x:c r="G196" s="8"/>
+      <x:c r="H196" s="8"/>
+      <x:c r="I196" s="8"/>
+      <x:c r="J196" s="8"/>
+      <x:c r="K196" s="8"/>
+      <x:c r="L196" s="8"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="8"/>
+      <x:c r="B197" s="8"/>
+      <x:c r="C197" s="8"/>
+      <x:c r="D197" s="8"/>
+      <x:c r="E197" s="8"/>
+      <x:c r="F197" s="8"/>
+      <x:c r="G197" s="8"/>
+      <x:c r="H197" s="8"/>
+      <x:c r="I197" s="8"/>
+      <x:c r="J197" s="8"/>
+      <x:c r="K197" s="8"/>
+      <x:c r="L197" s="8"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="8"/>
+      <x:c r="B198" s="8"/>
+      <x:c r="C198" s="8"/>
+      <x:c r="D198" s="8"/>
+      <x:c r="E198" s="8"/>
+      <x:c r="F198" s="8"/>
+      <x:c r="G198" s="8"/>
+      <x:c r="H198" s="8"/>
+      <x:c r="I198" s="8"/>
+      <x:c r="J198" s="8"/>
+      <x:c r="K198" s="8"/>
+      <x:c r="L198" s="8"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="8"/>
+      <x:c r="B199" s="8"/>
+      <x:c r="C199" s="8"/>
+      <x:c r="D199" s="8"/>
+      <x:c r="E199" s="8"/>
+      <x:c r="F199" s="8"/>
+      <x:c r="G199" s="8"/>
+      <x:c r="H199" s="8"/>
+      <x:c r="I199" s="8"/>
+      <x:c r="J199" s="8"/>
+      <x:c r="K199" s="8"/>
+      <x:c r="L199" s="8"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" s="8"/>
+      <x:c r="B200" s="8"/>
+      <x:c r="C200" s="8"/>
+      <x:c r="D200" s="8"/>
+      <x:c r="E200" s="8"/>
+      <x:c r="F200" s="8"/>
+      <x:c r="G200" s="8"/>
+      <x:c r="H200" s="8"/>
+      <x:c r="I200" s="8"/>
+      <x:c r="J200" s="8"/>
+      <x:c r="K200" s="8"/>
+      <x:c r="L200" s="8"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3068,9 +3708,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="44" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3429,7 +4069,7 @@
         <x:v>nfc_credential_provisioning</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>2026092202</x:v>
+        <x:v>2026092502</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>English</x:v>

</xml_diff>

<commit_message>
Release v2.11.0: NFC credential expiry and staged provisioning
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/nfc/example_odk_nfc_credential_provisioning.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/nfc/example_odk_nfc_credential_provisioning.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rdd4766b1ab16440e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R06fac21d64274738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Redd2dec1f6a34994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Ra8eee4f07ceb4088"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R34c2558039c04d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Re299aaf4d89c4bba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -320,13 +320,17 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
-        <x:v>start</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
-        <x:v>start</x:v>
-      </x:c>
-      <x:c r="C2" s="8"/>
-      <x:c r="D2" s="8"/>
+        <x:v>introduction</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>Provision an NFC credential</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="str">
+        <x:v>Enter the minimum provisioning inputs, then complete the PIN and NFC steps in MethodMesh.</x:v>
+      </x:c>
       <x:c r="E2" s="8"/>
       <x:c r="F2" s="8"/>
       <x:c r="G2" s="8"/>
@@ -339,17 +343,27 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
-        <x:v>end</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>end</x:v>
-      </x:c>
-      <x:c r="C3" s="8"/>
-      <x:c r="D3" s="8"/>
-      <x:c r="E3" s="8"/>
+        <x:v>credential_subject_id_input</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>Credential subject ID</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="str">
+        <x:v>Stable pseudonymous ID written into the encrypted credential.</x:v>
+      </x:c>
+      <x:c r="E3" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
       <x:c r="F3" s="8"/>
-      <x:c r="G3" s="8"/>
-      <x:c r="H3" s="8"/>
+      <x:c r="G3" s="8" t="str">
+        <x:v>string-length(.) &gt;= 2 and string-length(.) &lt;= 64</x:v>
+      </x:c>
+      <x:c r="H3" s="8" t="str">
+        <x:v>Use a stable ID between 2 and 64 characters.</x:v>
+      </x:c>
       <x:c r="I3" s="8"/>
       <x:c r="J3" s="8"/>
       <x:c r="K3" s="8"/>
@@ -358,18 +372,20 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="8" t="str">
-        <x:v>note</x:v>
+        <x:v>date</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>introduction</x:v>
+        <x:v>valid_until_date</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
-        <x:v>Provision a MethodMesh NFC credential</x:v>
+        <x:v>Credential valid until</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str">
-        <x:v>This example models a real study credential registry. Personal/study identity is stored in this ODK submission (and later central study systems), while MethodMesh handles the NFC cryptographic credential and returns the actual provisioning-device issuer identity.</x:v>
-      </x:c>
-      <x:c r="E4" s="8"/>
+        <x:v>Inclusive calendar date. MethodMesh converts this to the following UTC midnight.</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
       <x:c r="F4" s="8"/>
       <x:c r="G4" s="8"/>
       <x:c r="H4" s="8"/>
@@ -381,22 +397,24 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
-        <x:v>begin group</x:v>
+        <x:v>calculate</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>study_context</x:v>
-      </x:c>
-      <x:c r="C5" s="8" t="str">
-        <x:v>Credential holder and study context</x:v>
-      </x:c>
-      <x:c r="D5" s="8"/>
+        <x:v>valid_until_date_iso</x:v>
+      </x:c>
+      <x:c r="C5" s="8"/>
+      <x:c r="D5" s="8" t="str">
+        <x:v>Normalized ISO date passed to MethodMesh.</x:v>
+      </x:c>
       <x:c r="E5" s="8"/>
       <x:c r="F5" s="8"/>
       <x:c r="G5" s="8"/>
       <x:c r="H5" s="8"/>
-      <x:c r="I5" s="8"/>
+      <x:c r="I5" s="8" t="str">
+        <x:v>format-date(${valid_until_date}, '%Y-%m-%d')</x:v>
+      </x:c>
       <x:c r="J5" s="8" t="str">
-        <x:v>field-list</x:v>
+        <x:v>hidden</x:v>
       </x:c>
       <x:c r="K5" s="8"/>
       <x:c r="L5" s="8"/>
@@ -404,44 +422,44 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one pin_length</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>study_id</x:v>
+        <x:v>pin_length_input</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>Study / protocol ID</x:v>
+        <x:v>PIN length</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>Stable study or protocol code.</x:v>
+        <x:v>The PIN is entered only inside MethodMesh.</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="F6" s="8"/>
-      <x:c r="G6" s="8" t="str">
-        <x:v>string-length(.) &lt;= 64</x:v>
-      </x:c>
-      <x:c r="H6" s="8" t="str">
-        <x:v>Use a study ID of 64 characters or fewer.</x:v>
-      </x:c>
+      <x:c r="G6" s="8"/>
+      <x:c r="H6" s="8"/>
       <x:c r="I6" s="8"/>
       <x:c r="J6" s="8"/>
-      <x:c r="K6" s="8"/>
+      <x:c r="K6" s="8" t="str">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="L6" s="8"/>
       <x:c r="M6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8" t="str">
-        <x:v>select_one holder_type</x:v>
+        <x:v>select_one overwrite_policy</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>holder_type</x:v>
+        <x:v>overwrite_policy_input</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
-        <x:v>Credential holder type</x:v>
-      </x:c>
-      <x:c r="D7" s="8"/>
+        <x:v>Existing card content</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>Empty only is the safe default; Replace is explicit.</x:v>
+      </x:c>
       <x:c r="E7" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
@@ -450,37 +468,37 @@
       <x:c r="H7" s="8"/>
       <x:c r="I7" s="8"/>
       <x:c r="J7" s="8"/>
-      <x:c r="K7" s="8"/>
+      <x:c r="K7" s="8" t="str">
+        <x:v>empty_only</x:v>
+      </x:c>
       <x:c r="L7" s="8"/>
       <x:c r="M7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>begin group</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>credential_subject_id_input</x:v>
+        <x:v>run_nfc_credential_provisioning</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>Credential subject / registry ID</x:v>
+        <x:v>Write and verify NFC credential</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
-        <x:v>Use a short stable pseudonymous ID, not the person's name or email. This is passed to MethodMesh and recovered after successful PIN verification.</x:v>
-      </x:c>
-      <x:c r="E8" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Tap the card when prompted in MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E8" s="8"/>
       <x:c r="F8" s="8"/>
-      <x:c r="G8" s="8" t="str">
-        <x:v>string-length(.) &gt;= 2 and string-length(.) &lt;= 64</x:v>
-      </x:c>
-      <x:c r="H8" s="8" t="str">
-        <x:v>Use a stable ID between 2 and 64 characters.</x:v>
-      </x:c>
+      <x:c r="G8" s="8"/>
+      <x:c r="H8" s="8"/>
       <x:c r="I8" s="8"/>
-      <x:c r="J8" s="8"/>
+      <x:c r="J8" s="8" t="str">
+        <x:v>field-list</x:v>
+      </x:c>
       <x:c r="K8" s="8"/>
-      <x:c r="L8" s="8"/>
+      <x:c r="L8" s="8" t="str">
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_valid_until_date=${valid_until_date_iso},input_overwrite_policy=${overwrite_policy_input},input_payload_mode='FULL',return_mode='flat')</x:v>
+      </x:c>
       <x:c r="M8"/>
     </x:row>
     <x:row r="9">
@@ -488,45 +506,47 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>holder_display_name</x:v>
+        <x:v>methodmesh_status</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>Name / display name</x:v>
+        <x:v>MethodMesh status</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
-        <x:v>Registry field only: retained in ODK/Sentinel and not sent to MethodMesh or written to the card.</x:v>
-      </x:c>
-      <x:c r="E9" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E9" s="8"/>
       <x:c r="F9" s="8"/>
       <x:c r="G9" s="8"/>
       <x:c r="H9" s="8"/>
       <x:c r="I9" s="8"/>
-      <x:c r="J9" s="8"/>
+      <x:c r="J9" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="K9" s="8"/>
       <x:c r="L9" s="8"/>
       <x:c r="M9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
-        <x:v>select_one credential_role</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>holder_role</x:v>
+        <x:v>credential_id</x:v>
       </x:c>
       <x:c r="C10" s="8" t="str">
-        <x:v>Study role</x:v>
-      </x:c>
-      <x:c r="D10" s="8"/>
-      <x:c r="E10" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Credential ID</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E10" s="8"/>
       <x:c r="F10" s="8"/>
       <x:c r="G10" s="8"/>
       <x:c r="H10" s="8"/>
       <x:c r="I10" s="8"/>
-      <x:c r="J10" s="8"/>
+      <x:c r="J10" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="K10" s="8"/>
       <x:c r="L10" s="8"/>
       <x:c r="M10"/>
@@ -536,22 +556,22 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>holder_role_other</x:v>
+        <x:v>credential_subject_id</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
-        <x:v>Other role</x:v>
-      </x:c>
-      <x:c r="D11" s="8"/>
-      <x:c r="E11" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="F11" s="8" t="str">
-        <x:v>${holder_role} = 'other'</x:v>
-      </x:c>
+        <x:v>Credential subject ID returned</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E11" s="8"/>
+      <x:c r="F11" s="8"/>
       <x:c r="G11" s="8"/>
       <x:c r="H11" s="8"/>
       <x:c r="I11" s="8"/>
-      <x:c r="J11" s="8"/>
+      <x:c r="J11" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="K11" s="8"/>
       <x:c r="L11" s="8"/>
       <x:c r="M11"/>
@@ -561,17 +581,15 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>site_code</x:v>
+        <x:v>valid_until_iso</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
-        <x:v>Site / location code</x:v>
+        <x:v>Credential valid until (UTC)</x:v>
       </x:c>
       <x:c r="D12" s="8" t="str">
-        <x:v>Study site, clinic, laboratory or operating location.</x:v>
-      </x:c>
-      <x:c r="E12" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Authenticated exclusive expiry instant returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E12" s="8"/>
       <x:c r="F12" s="8"/>
       <x:c r="G12" s="8"/>
       <x:c r="H12" s="8"/>
@@ -586,13 +604,13 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
-        <x:v>organisation</x:v>
+        <x:v>provision_success</x:v>
       </x:c>
       <x:c r="C13" s="8" t="str">
-        <x:v>Organisation / team</x:v>
+        <x:v>Provisioning succeeded</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
-        <x:v>Optional employing organisation or study team.</x:v>
+        <x:v>Returned by MethodMesh.</x:v>
       </x:c>
       <x:c r="E13" s="8"/>
       <x:c r="F13" s="8"/>
@@ -606,52 +624,46 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
-        <x:v>date</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B14" s="8" t="str">
-        <x:v>valid_from_date</x:v>
+        <x:v>provision_message</x:v>
       </x:c>
       <x:c r="C14" s="8" t="str">
-        <x:v>Credential valid from</x:v>
+        <x:v>Provisioning result</x:v>
       </x:c>
       <x:c r="D14" s="8" t="str">
-        <x:v>Governance/registry validity start. Under the current ROSC1 contract this date is not encoded into the NFC credential itself.</x:v>
-      </x:c>
-      <x:c r="E14" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Human-readable write/verification result.</x:v>
+      </x:c>
+      <x:c r="E14" s="8"/>
       <x:c r="F14" s="8"/>
       <x:c r="G14" s="8"/>
       <x:c r="H14" s="8"/>
       <x:c r="I14" s="8"/>
-      <x:c r="J14" s="8"/>
+      <x:c r="J14" s="8" t="str">
+        <x:v>multiline</x:v>
+      </x:c>
       <x:c r="K14" s="8"/>
       <x:c r="L14" s="8"/>
       <x:c r="M14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
-        <x:v>date</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>valid_until_date</x:v>
+        <x:v>write_verified</x:v>
       </x:c>
       <x:c r="C15" s="8" t="str">
-        <x:v>Credential valid until</x:v>
+        <x:v>Write verified</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
-        <x:v>Governance/registry validity end. Under the current ROSC1 contract this date is not encoded into the NFC credential itself.</x:v>
-      </x:c>
-      <x:c r="E15" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>True only after the deliberate verification tap.</x:v>
+      </x:c>
+      <x:c r="E15" s="8"/>
       <x:c r="F15" s="8"/>
-      <x:c r="G15" s="8" t="str">
-        <x:v>. &gt;= ${valid_from_date}</x:v>
-      </x:c>
-      <x:c r="H15" s="8" t="str">
-        <x:v>End date must be on or after the start date.</x:v>
-      </x:c>
+      <x:c r="G15" s="8"/>
+      <x:c r="H15" s="8"/>
       <x:c r="I15" s="8"/>
       <x:c r="J15" s="8"/>
       <x:c r="K15" s="8"/>
@@ -663,45 +675,47 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B16" s="8" t="str">
-        <x:v>authorised_by</x:v>
+        <x:v>written_message_hash</x:v>
       </x:c>
       <x:c r="C16" s="8" t="str">
-        <x:v>Authorised by</x:v>
+        <x:v>Written message SHA-256</x:v>
       </x:c>
       <x:c r="D16" s="8" t="str">
-        <x:v>Name or identifier of the person authorising issuance.</x:v>
-      </x:c>
-      <x:c r="E16" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Returned by MethodMesh for audit confirmation.</x:v>
+      </x:c>
+      <x:c r="E16" s="8"/>
       <x:c r="F16" s="8"/>
       <x:c r="G16" s="8"/>
       <x:c r="H16" s="8"/>
       <x:c r="I16" s="8"/>
-      <x:c r="J16" s="8"/>
+      <x:c r="J16" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="K16" s="8"/>
       <x:c r="L16" s="8"/>
       <x:c r="M16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
-        <x:v>select_one provision_reason</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B17" s="8" t="str">
-        <x:v>provision_reason</x:v>
+        <x:v>issuer_key_id</x:v>
       </x:c>
       <x:c r="C17" s="8" t="str">
-        <x:v>Reason for issuing credential</x:v>
-      </x:c>
-      <x:c r="D17" s="8"/>
-      <x:c r="E17" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Issuer key ID</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="str">
+        <x:v>Provisioning-device identity evidence.</x:v>
+      </x:c>
+      <x:c r="E17" s="8"/>
       <x:c r="F17" s="8"/>
       <x:c r="G17" s="8"/>
       <x:c r="H17" s="8"/>
       <x:c r="I17" s="8"/>
-      <x:c r="J17" s="8"/>
+      <x:c r="J17" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="K17" s="8"/>
       <x:c r="L17" s="8"/>
       <x:c r="M17"/>
@@ -711,22 +725,22 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B18" s="8" t="str">
-        <x:v>provision_reason_other</x:v>
+        <x:v>issuer_public_key_fingerprint_sha256</x:v>
       </x:c>
       <x:c r="C18" s="8" t="str">
-        <x:v>Other issuance reason</x:v>
-      </x:c>
-      <x:c r="D18" s="8"/>
-      <x:c r="E18" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="F18" s="8" t="str">
-        <x:v>${provision_reason} = 'other'</x:v>
-      </x:c>
+        <x:v>Issuer public key fingerprint</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>Provisioning-device identity evidence for Sentinel reconciliation.</x:v>
+      </x:c>
+      <x:c r="E18" s="8"/>
+      <x:c r="F18" s="8"/>
       <x:c r="G18" s="8"/>
       <x:c r="H18" s="8"/>
       <x:c r="I18" s="8"/>
-      <x:c r="J18" s="8"/>
+      <x:c r="J18" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="K18" s="8"/>
       <x:c r="L18" s="8"/>
       <x:c r="M18"/>
@@ -736,32 +750,30 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B19" s="8" t="str">
-        <x:v>registry_notes</x:v>
+        <x:v>methodmesh_full_json</x:v>
       </x:c>
       <x:c r="C19" s="8" t="str">
-        <x:v>Registry notes</x:v>
+        <x:v>MethodMesh FULL JSON (technical)</x:v>
       </x:c>
       <x:c r="D19" s="8" t="str">
-        <x:v>Optional study administration notes. Do not enter the PIN.</x:v>
+        <x:v>Complete execution envelope retained as one field for downstream audit and integration.</x:v>
       </x:c>
       <x:c r="E19" s="8"/>
       <x:c r="F19" s="8"/>
       <x:c r="G19" s="8"/>
       <x:c r="H19" s="8"/>
       <x:c r="I19" s="8"/>
-      <x:c r="J19" s="8" t="str">
-        <x:v>multiline</x:v>
-      </x:c>
+      <x:c r="J19" s="8"/>
       <x:c r="K19" s="8"/>
       <x:c r="L19" s="8"/>
       <x:c r="M19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
-        <x:v>calculate</x:v>
+        <x:v>end group</x:v>
       </x:c>
       <x:c r="B20" s="8" t="str">
-        <x:v>credential_registry_key</x:v>
+        <x:v>run_nfc_credential_provisioning_end</x:v>
       </x:c>
       <x:c r="C20" s="8"/>
       <x:c r="D20" s="8"/>
@@ -769,9 +781,7 @@
       <x:c r="F20" s="8"/>
       <x:c r="G20" s="8"/>
       <x:c r="H20" s="8"/>
-      <x:c r="I20" s="8" t="str">
-        <x:v>concat(${study_id}, '|', ${credential_subject_id_input})</x:v>
-      </x:c>
+      <x:c r="I20" s="8"/>
       <x:c r="J20" s="8"/>
       <x:c r="K20" s="8"/>
       <x:c r="L20" s="8"/>
@@ -779,15 +789,21 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8" t="str">
-        <x:v>end group</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="B21" s="8" t="str">
-        <x:v>study_context_end</x:v>
-      </x:c>
-      <x:c r="C21" s="8"/>
-      <x:c r="D21" s="8"/>
+        <x:v>provision_summary</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>Credential provisioning result</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>Credential ${credential_id}; valid until ${valid_until_iso}; status ${methodmesh_status}; write verified ${write_verified}; result ${provision_message}.</x:v>
+      </x:c>
       <x:c r="E21" s="8"/>
-      <x:c r="F21" s="8"/>
+      <x:c r="F21" s="8" t="str">
+        <x:v>${methodmesh_status} != ''</x:v>
+      </x:c>
       <x:c r="G21" s="8"/>
       <x:c r="H21" s="8"/>
       <x:c r="I21" s="8"/>
@@ -797,95 +813,55 @@
       <x:c r="M21"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="8" t="str">
-        <x:v>begin group</x:v>
-      </x:c>
-      <x:c r="B22" s="8" t="str">
-        <x:v>credential_options</x:v>
-      </x:c>
-      <x:c r="C22" s="8" t="str">
-        <x:v>Credential security options</x:v>
-      </x:c>
+      <x:c r="A22" s="8"/>
+      <x:c r="B22" s="8"/>
+      <x:c r="C22" s="8"/>
       <x:c r="D22" s="8"/>
       <x:c r="E22" s="8"/>
       <x:c r="F22" s="8"/>
       <x:c r="G22" s="8"/>
       <x:c r="H22" s="8"/>
       <x:c r="I22" s="8"/>
-      <x:c r="J22" s="8" t="str">
-        <x:v>field-list</x:v>
-      </x:c>
+      <x:c r="J22" s="8"/>
       <x:c r="K22" s="8"/>
       <x:c r="L22" s="8"/>
       <x:c r="M22"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="8" t="str">
-        <x:v>select_one pin_length</x:v>
-      </x:c>
-      <x:c r="B23" s="8" t="str">
-        <x:v>pin_length_input</x:v>
-      </x:c>
-      <x:c r="C23" s="8" t="str">
-        <x:v>PIN length</x:v>
-      </x:c>
-      <x:c r="D23" s="8" t="str">
-        <x:v>The PIN itself is entered only inside MethodMesh and is never returned to ODK.</x:v>
-      </x:c>
-      <x:c r="E23" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+      <x:c r="A23" s="8"/>
+      <x:c r="B23" s="8"/>
+      <x:c r="C23" s="8"/>
+      <x:c r="D23" s="8"/>
+      <x:c r="E23" s="8"/>
       <x:c r="F23" s="8"/>
       <x:c r="G23" s="8"/>
       <x:c r="H23" s="8"/>
       <x:c r="I23" s="8"/>
       <x:c r="J23" s="8"/>
-      <x:c r="K23" s="8" t="str">
-        <x:v>6</x:v>
-      </x:c>
+      <x:c r="K23" s="8"/>
       <x:c r="L23" s="8"/>
       <x:c r="M23"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="8" t="str">
-        <x:v>select_one overwrite_policy</x:v>
-      </x:c>
-      <x:c r="B24" s="8" t="str">
-        <x:v>overwrite_policy_input</x:v>
-      </x:c>
-      <x:c r="C24" s="8" t="str">
-        <x:v>NFC overwrite policy</x:v>
-      </x:c>
-      <x:c r="D24" s="8" t="str">
-        <x:v>Use empty_only for new cards. Replace should only be used when intentionally reissuing/replacing a credential.</x:v>
-      </x:c>
-      <x:c r="E24" s="8" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+      <x:c r="A24" s="8"/>
+      <x:c r="B24" s="8"/>
+      <x:c r="C24" s="8"/>
+      <x:c r="D24" s="8"/>
+      <x:c r="E24" s="8"/>
       <x:c r="F24" s="8"/>
       <x:c r="G24" s="8"/>
       <x:c r="H24" s="8"/>
       <x:c r="I24" s="8"/>
       <x:c r="J24" s="8"/>
-      <x:c r="K24" s="8" t="str">
-        <x:v>empty_only</x:v>
-      </x:c>
+      <x:c r="K24" s="8"/>
       <x:c r="L24" s="8"/>
       <x:c r="M24"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="8" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="B25" s="8" t="str">
-        <x:v>security_note</x:v>
-      </x:c>
-      <x:c r="C25" s="8" t="str">
-        <x:v>PIN and credential secret handling</x:v>
-      </x:c>
-      <x:c r="D25" s="8" t="str">
-        <x:v>The operator enters and confirms the PIN inside MethodMesh. The form never stores the PIN, encryption key, random credential secret or encrypted envelope.</x:v>
-      </x:c>
+      <x:c r="A25" s="8"/>
+      <x:c r="B25" s="8"/>
+      <x:c r="C25" s="8"/>
+      <x:c r="D25" s="8"/>
       <x:c r="E25" s="8"/>
       <x:c r="F25" s="8"/>
       <x:c r="G25" s="8"/>
@@ -897,12 +873,8 @@
       <x:c r="M25"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="8" t="str">
-        <x:v>end group</x:v>
-      </x:c>
-      <x:c r="B26" s="8" t="str">
-        <x:v>credential_options_end</x:v>
-      </x:c>
+      <x:c r="A26" s="8"/>
+      <x:c r="B26" s="8"/>
       <x:c r="C26" s="8"/>
       <x:c r="D26" s="8"/>
       <x:c r="E26" s="8"/>
@@ -916,689 +888,413 @@
       <x:c r="M26"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="8" t="str">
-        <x:v>begin group</x:v>
-      </x:c>
-      <x:c r="B27" s="8" t="str">
-        <x:v>run_nfc_credential_provisioning</x:v>
-      </x:c>
-      <x:c r="C27" s="8" t="str">
-        <x:v>Write and verify NFC credential</x:v>
-      </x:c>
-      <x:c r="D27" s="8" t="str">
-        <x:v>Tap the credential card, complete the MethodMesh provisioning workflow, then Commit to return here.</x:v>
-      </x:c>
+      <x:c r="A27" s="8"/>
+      <x:c r="B27" s="8"/>
+      <x:c r="C27" s="8"/>
+      <x:c r="D27" s="8"/>
       <x:c r="E27" s="8"/>
       <x:c r="F27" s="8"/>
       <x:c r="G27" s="8"/>
       <x:c r="H27" s="8"/>
       <x:c r="I27" s="8"/>
-      <x:c r="J27" s="8" t="str">
-        <x:v>field-list</x:v>
-      </x:c>
+      <x:c r="J27" s="8"/>
       <x:c r="K27" s="8"/>
-      <x:c r="L27" s="8" t="str">
-        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_overwrite_policy=${overwrite_policy_input},input_payload_mode='FULL',return_mode='flat')</x:v>
-      </x:c>
+      <x:c r="L27" s="8"/>
       <x:c r="M27"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B28" s="8" t="str">
-        <x:v>methodmesh_execution_id</x:v>
-      </x:c>
-      <x:c r="C28" s="8" t="str">
-        <x:v>MethodMesh execution ID</x:v>
-      </x:c>
-      <x:c r="D28" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A28" s="8"/>
+      <x:c r="B28" s="8"/>
+      <x:c r="C28" s="8"/>
+      <x:c r="D28" s="8"/>
       <x:c r="E28" s="8"/>
       <x:c r="F28" s="8"/>
       <x:c r="G28" s="8"/>
       <x:c r="H28" s="8"/>
       <x:c r="I28" s="8"/>
-      <x:c r="J28" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J28" s="8"/>
       <x:c r="K28" s="8"/>
       <x:c r="L28" s="8"/>
       <x:c r="M28"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B29" s="8" t="str">
-        <x:v>methodmesh_status</x:v>
-      </x:c>
-      <x:c r="C29" s="8" t="str">
-        <x:v>MethodMesh status</x:v>
-      </x:c>
-      <x:c r="D29" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A29" s="8"/>
+      <x:c r="B29" s="8"/>
+      <x:c r="C29" s="8"/>
+      <x:c r="D29" s="8"/>
       <x:c r="E29" s="8"/>
       <x:c r="F29" s="8"/>
       <x:c r="G29" s="8"/>
       <x:c r="H29" s="8"/>
       <x:c r="I29" s="8"/>
-      <x:c r="J29" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J29" s="8"/>
       <x:c r="K29" s="8"/>
       <x:c r="L29" s="8"/>
       <x:c r="M29"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B30" s="8" t="str">
-        <x:v>credential_id</x:v>
-      </x:c>
-      <x:c r="C30" s="8" t="str">
-        <x:v>Credential ID</x:v>
-      </x:c>
-      <x:c r="D30" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A30" s="8"/>
+      <x:c r="B30" s="8"/>
+      <x:c r="C30" s="8"/>
+      <x:c r="D30" s="8"/>
       <x:c r="E30" s="8"/>
       <x:c r="F30" s="8"/>
       <x:c r="G30" s="8"/>
       <x:c r="H30" s="8"/>
       <x:c r="I30" s="8"/>
-      <x:c r="J30" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J30" s="8"/>
       <x:c r="K30" s="8"/>
       <x:c r="L30" s="8"/>
       <x:c r="M30"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B31" s="8" t="str">
-        <x:v>credential_subject_id</x:v>
-      </x:c>
-      <x:c r="C31" s="8" t="str">
-        <x:v>Credential subject ID returned</x:v>
-      </x:c>
-      <x:c r="D31" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A31" s="8"/>
+      <x:c r="B31" s="8"/>
+      <x:c r="C31" s="8"/>
+      <x:c r="D31" s="8"/>
       <x:c r="E31" s="8"/>
       <x:c r="F31" s="8"/>
       <x:c r="G31" s="8"/>
       <x:c r="H31" s="8"/>
       <x:c r="I31" s="8"/>
-      <x:c r="J31" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J31" s="8"/>
       <x:c r="K31" s="8"/>
       <x:c r="L31" s="8"/>
       <x:c r="M31"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="8" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="B32" s="8" t="str">
-        <x:v>pin_length</x:v>
-      </x:c>
-      <x:c r="C32" s="8" t="str">
-        <x:v>PIN length</x:v>
-      </x:c>
-      <x:c r="D32" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A32" s="8"/>
+      <x:c r="B32" s="8"/>
+      <x:c r="C32" s="8"/>
+      <x:c r="D32" s="8"/>
       <x:c r="E32" s="8"/>
       <x:c r="F32" s="8"/>
       <x:c r="G32" s="8"/>
       <x:c r="H32" s="8"/>
       <x:c r="I32" s="8"/>
-      <x:c r="J32" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J32" s="8"/>
       <x:c r="K32" s="8"/>
       <x:c r="L32" s="8"/>
       <x:c r="M32"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B33" s="8" t="str">
-        <x:v>credential_format_version</x:v>
-      </x:c>
-      <x:c r="C33" s="8" t="str">
-        <x:v>Credential format version</x:v>
-      </x:c>
-      <x:c r="D33" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A33" s="8"/>
+      <x:c r="B33" s="8"/>
+      <x:c r="C33" s="8"/>
+      <x:c r="D33" s="8"/>
       <x:c r="E33" s="8"/>
       <x:c r="F33" s="8"/>
       <x:c r="G33" s="8"/>
       <x:c r="H33" s="8"/>
       <x:c r="I33" s="8"/>
-      <x:c r="J33" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J33" s="8"/>
       <x:c r="K33" s="8"/>
       <x:c r="L33" s="8"/>
       <x:c r="M33"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B34" s="8" t="str">
-        <x:v>key_derivation</x:v>
-      </x:c>
-      <x:c r="C34" s="8" t="str">
-        <x:v>Key derivation</x:v>
-      </x:c>
-      <x:c r="D34" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A34" s="8"/>
+      <x:c r="B34" s="8"/>
+      <x:c r="C34" s="8"/>
+      <x:c r="D34" s="8"/>
       <x:c r="E34" s="8"/>
       <x:c r="F34" s="8"/>
       <x:c r="G34" s="8"/>
       <x:c r="H34" s="8"/>
       <x:c r="I34" s="8"/>
-      <x:c r="J34" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J34" s="8"/>
       <x:c r="K34" s="8"/>
       <x:c r="L34" s="8"/>
       <x:c r="M34"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B35" s="8" t="str">
-        <x:v>credential_issued_time_iso</x:v>
-      </x:c>
-      <x:c r="C35" s="8" t="str">
-        <x:v>Credential issued time</x:v>
-      </x:c>
-      <x:c r="D35" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A35" s="8"/>
+      <x:c r="B35" s="8"/>
+      <x:c r="C35" s="8"/>
+      <x:c r="D35" s="8"/>
       <x:c r="E35" s="8"/>
       <x:c r="F35" s="8"/>
       <x:c r="G35" s="8"/>
       <x:c r="H35" s="8"/>
       <x:c r="I35" s="8"/>
-      <x:c r="J35" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J35" s="8"/>
       <x:c r="K35" s="8"/>
       <x:c r="L35" s="8"/>
       <x:c r="M35"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B36" s="8" t="str">
-        <x:v>credential_envelope_hash</x:v>
-      </x:c>
-      <x:c r="C36" s="8" t="str">
-        <x:v>Credential envelope SHA-256</x:v>
-      </x:c>
-      <x:c r="D36" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A36" s="8"/>
+      <x:c r="B36" s="8"/>
+      <x:c r="C36" s="8"/>
+      <x:c r="D36" s="8"/>
       <x:c r="E36" s="8"/>
       <x:c r="F36" s="8"/>
       <x:c r="G36" s="8"/>
       <x:c r="H36" s="8"/>
       <x:c r="I36" s="8"/>
-      <x:c r="J36" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J36" s="8"/>
       <x:c r="K36" s="8"/>
       <x:c r="L36" s="8"/>
       <x:c r="M36"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B37" s="8" t="str">
-        <x:v>credential_secret_hash</x:v>
-      </x:c>
-      <x:c r="C37" s="8" t="str">
-        <x:v>Credential secret SHA-256</x:v>
-      </x:c>
-      <x:c r="D37" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A37" s="8"/>
+      <x:c r="B37" s="8"/>
+      <x:c r="C37" s="8"/>
+      <x:c r="D37" s="8"/>
       <x:c r="E37" s="8"/>
       <x:c r="F37" s="8"/>
       <x:c r="G37" s="8"/>
       <x:c r="H37" s="8"/>
       <x:c r="I37" s="8"/>
-      <x:c r="J37" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J37" s="8"/>
       <x:c r="K37" s="8"/>
       <x:c r="L37" s="8"/>
       <x:c r="M37"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B38" s="8" t="str">
-        <x:v>issuer_key_id</x:v>
-      </x:c>
-      <x:c r="C38" s="8" t="str">
-        <x:v>Issuer key ID</x:v>
-      </x:c>
-      <x:c r="D38" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A38" s="8"/>
+      <x:c r="B38" s="8"/>
+      <x:c r="C38" s="8"/>
+      <x:c r="D38" s="8"/>
       <x:c r="E38" s="8"/>
       <x:c r="F38" s="8"/>
       <x:c r="G38" s="8"/>
       <x:c r="H38" s="8"/>
       <x:c r="I38" s="8"/>
-      <x:c r="J38" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J38" s="8"/>
       <x:c r="K38" s="8"/>
       <x:c r="L38" s="8"/>
       <x:c r="M38"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B39" s="8" t="str">
-        <x:v>issuer_public_key_fingerprint_sha256</x:v>
-      </x:c>
-      <x:c r="C39" s="8" t="str">
-        <x:v>Issuer public key SHA-256 fingerprint</x:v>
-      </x:c>
-      <x:c r="D39" s="8" t="str">
-        <x:v>Canonical full 64-character provisioning-device identity derived by MethodMesh from the issuer public key.</x:v>
-      </x:c>
+      <x:c r="A39" s="8"/>
+      <x:c r="B39" s="8"/>
+      <x:c r="C39" s="8"/>
+      <x:c r="D39" s="8"/>
       <x:c r="E39" s="8"/>
       <x:c r="F39" s="8"/>
       <x:c r="G39" s="8"/>
       <x:c r="H39" s="8"/>
       <x:c r="I39" s="8"/>
-      <x:c r="J39" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J39" s="8"/>
       <x:c r="K39" s="8"/>
       <x:c r="L39" s="8"/>
       <x:c r="M39"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B40" s="8" t="str">
-        <x:v>issuer_public_key_base64</x:v>
-      </x:c>
-      <x:c r="C40" s="8" t="str">
-        <x:v>Issuer public key</x:v>
-      </x:c>
-      <x:c r="D40" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A40" s="8"/>
+      <x:c r="B40" s="8"/>
+      <x:c r="C40" s="8"/>
+      <x:c r="D40" s="8"/>
       <x:c r="E40" s="8"/>
       <x:c r="F40" s="8"/>
       <x:c r="G40" s="8"/>
       <x:c r="H40" s="8"/>
       <x:c r="I40" s="8"/>
-      <x:c r="J40" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J40" s="8"/>
       <x:c r="K40" s="8"/>
       <x:c r="L40" s="8"/>
       <x:c r="M40"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B41" s="8" t="str">
-        <x:v>issuer_signature_algorithm</x:v>
-      </x:c>
-      <x:c r="C41" s="8" t="str">
-        <x:v>Issuer signature algorithm</x:v>
-      </x:c>
-      <x:c r="D41" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A41" s="8"/>
+      <x:c r="B41" s="8"/>
+      <x:c r="C41" s="8"/>
+      <x:c r="D41" s="8"/>
       <x:c r="E41" s="8"/>
       <x:c r="F41" s="8"/>
       <x:c r="G41" s="8"/>
       <x:c r="H41" s="8"/>
       <x:c r="I41" s="8"/>
-      <x:c r="J41" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J41" s="8"/>
       <x:c r="K41" s="8"/>
       <x:c r="L41" s="8"/>
       <x:c r="M41"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B42" s="8" t="str">
-        <x:v>provision_success</x:v>
-      </x:c>
-      <x:c r="C42" s="8" t="str">
-        <x:v>Provision success</x:v>
-      </x:c>
-      <x:c r="D42" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A42" s="8"/>
+      <x:c r="B42" s="8"/>
+      <x:c r="C42" s="8"/>
+      <x:c r="D42" s="8"/>
       <x:c r="E42" s="8"/>
       <x:c r="F42" s="8"/>
       <x:c r="G42" s="8"/>
       <x:c r="H42" s="8"/>
       <x:c r="I42" s="8"/>
-      <x:c r="J42" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J42" s="8"/>
       <x:c r="K42" s="8"/>
       <x:c r="L42" s="8"/>
       <x:c r="M42"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B43" s="8" t="str">
-        <x:v>provision_message</x:v>
-      </x:c>
-      <x:c r="C43" s="8" t="str">
-        <x:v>Provisioning result</x:v>
-      </x:c>
-      <x:c r="D43" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A43" s="8"/>
+      <x:c r="B43" s="8"/>
+      <x:c r="C43" s="8"/>
+      <x:c r="D43" s="8"/>
       <x:c r="E43" s="8"/>
       <x:c r="F43" s="8"/>
       <x:c r="G43" s="8"/>
       <x:c r="H43" s="8"/>
       <x:c r="I43" s="8"/>
-      <x:c r="J43" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J43" s="8"/>
       <x:c r="K43" s="8"/>
       <x:c r="L43" s="8"/>
       <x:c r="M43"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B44" s="8" t="str">
-        <x:v>provisioned_time_iso</x:v>
-      </x:c>
-      <x:c r="C44" s="8" t="str">
-        <x:v>Provisioned time</x:v>
-      </x:c>
-      <x:c r="D44" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A44" s="8"/>
+      <x:c r="B44" s="8"/>
+      <x:c r="C44" s="8"/>
+      <x:c r="D44" s="8"/>
       <x:c r="E44" s="8"/>
       <x:c r="F44" s="8"/>
       <x:c r="G44" s="8"/>
       <x:c r="H44" s="8"/>
       <x:c r="I44" s="8"/>
-      <x:c r="J44" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J44" s="8"/>
       <x:c r="K44" s="8"/>
       <x:c r="L44" s="8"/>
       <x:c r="M44"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B45" s="8" t="str">
-        <x:v>write_record_type</x:v>
-      </x:c>
-      <x:c r="C45" s="8" t="str">
-        <x:v>NFC write record type</x:v>
-      </x:c>
-      <x:c r="D45" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A45" s="8"/>
+      <x:c r="B45" s="8"/>
+      <x:c r="C45" s="8"/>
+      <x:c r="D45" s="8"/>
       <x:c r="E45" s="8"/>
       <x:c r="F45" s="8"/>
       <x:c r="G45" s="8"/>
       <x:c r="H45" s="8"/>
       <x:c r="I45" s="8"/>
-      <x:c r="J45" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J45" s="8"/>
       <x:c r="K45" s="8"/>
       <x:c r="L45" s="8"/>
       <x:c r="M45"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="8" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="B46" s="8" t="str">
-        <x:v>write_size_bytes</x:v>
-      </x:c>
-      <x:c r="C46" s="8" t="str">
-        <x:v>NFC write size (bytes)</x:v>
-      </x:c>
-      <x:c r="D46" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A46" s="8"/>
+      <x:c r="B46" s="8"/>
+      <x:c r="C46" s="8"/>
+      <x:c r="D46" s="8"/>
       <x:c r="E46" s="8"/>
       <x:c r="F46" s="8"/>
       <x:c r="G46" s="8"/>
       <x:c r="H46" s="8"/>
       <x:c r="I46" s="8"/>
-      <x:c r="J46" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J46" s="8"/>
       <x:c r="K46" s="8"/>
       <x:c r="L46" s="8"/>
       <x:c r="M46"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B47" s="8" t="str">
-        <x:v>overwrite_policy</x:v>
-      </x:c>
-      <x:c r="C47" s="8" t="str">
-        <x:v>Applied overwrite policy</x:v>
-      </x:c>
-      <x:c r="D47" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A47" s="8"/>
+      <x:c r="B47" s="8"/>
+      <x:c r="C47" s="8"/>
+      <x:c r="D47" s="8"/>
       <x:c r="E47" s="8"/>
       <x:c r="F47" s="8"/>
       <x:c r="G47" s="8"/>
       <x:c r="H47" s="8"/>
       <x:c r="I47" s="8"/>
-      <x:c r="J47" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J47" s="8"/>
       <x:c r="K47" s="8"/>
       <x:c r="L47" s="8"/>
       <x:c r="M47"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B48" s="8" t="str">
-        <x:v>previous_message_hash</x:v>
-      </x:c>
-      <x:c r="C48" s="8" t="str">
-        <x:v>Previous NFC message SHA-256</x:v>
-      </x:c>
-      <x:c r="D48" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A48" s="8"/>
+      <x:c r="B48" s="8"/>
+      <x:c r="C48" s="8"/>
+      <x:c r="D48" s="8"/>
       <x:c r="E48" s="8"/>
       <x:c r="F48" s="8"/>
       <x:c r="G48" s="8"/>
       <x:c r="H48" s="8"/>
       <x:c r="I48" s="8"/>
-      <x:c r="J48" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J48" s="8"/>
       <x:c r="K48" s="8"/>
       <x:c r="L48" s="8"/>
       <x:c r="M48"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B49" s="8" t="str">
-        <x:v>written_message_hash</x:v>
-      </x:c>
-      <x:c r="C49" s="8" t="str">
-        <x:v>Written NFC message SHA-256</x:v>
-      </x:c>
-      <x:c r="D49" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A49" s="8"/>
+      <x:c r="B49" s="8"/>
+      <x:c r="C49" s="8"/>
+      <x:c r="D49" s="8"/>
       <x:c r="E49" s="8"/>
       <x:c r="F49" s="8"/>
       <x:c r="G49" s="8"/>
       <x:c r="H49" s="8"/>
       <x:c r="I49" s="8"/>
-      <x:c r="J49" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J49" s="8"/>
       <x:c r="K49" s="8"/>
       <x:c r="L49" s="8"/>
       <x:c r="M49"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B50" s="8" t="str">
-        <x:v>write_verified</x:v>
-      </x:c>
-      <x:c r="C50" s="8" t="str">
-        <x:v>NFC write verified</x:v>
-      </x:c>
-      <x:c r="D50" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A50" s="8"/>
+      <x:c r="B50" s="8"/>
+      <x:c r="C50" s="8"/>
+      <x:c r="D50" s="8"/>
       <x:c r="E50" s="8"/>
       <x:c r="F50" s="8"/>
       <x:c r="G50" s="8"/>
       <x:c r="H50" s="8"/>
       <x:c r="I50" s="8"/>
-      <x:c r="J50" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J50" s="8"/>
       <x:c r="K50" s="8"/>
       <x:c r="L50" s="8"/>
       <x:c r="M50"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B51" s="8" t="str">
-        <x:v>tag_uid_hex</x:v>
-      </x:c>
-      <x:c r="C51" s="8" t="str">
-        <x:v>NFC tag UID</x:v>
-      </x:c>
-      <x:c r="D51" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A51" s="8"/>
+      <x:c r="B51" s="8"/>
+      <x:c r="C51" s="8"/>
+      <x:c r="D51" s="8"/>
       <x:c r="E51" s="8"/>
       <x:c r="F51" s="8"/>
       <x:c r="G51" s="8"/>
       <x:c r="H51" s="8"/>
       <x:c r="I51" s="8"/>
-      <x:c r="J51" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J51" s="8"/>
       <x:c r="K51" s="8"/>
       <x:c r="L51" s="8"/>
       <x:c r="M51"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B52" s="8" t="str">
-        <x:v>verification_evidence_hash</x:v>
-      </x:c>
-      <x:c r="C52" s="8" t="str">
-        <x:v>Verification evidence SHA-256</x:v>
-      </x:c>
-      <x:c r="D52" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A52" s="8"/>
+      <x:c r="B52" s="8"/>
+      <x:c r="C52" s="8"/>
+      <x:c r="D52" s="8"/>
       <x:c r="E52" s="8"/>
       <x:c r="F52" s="8"/>
       <x:c r="G52" s="8"/>
       <x:c r="H52" s="8"/>
       <x:c r="I52" s="8"/>
-      <x:c r="J52" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J52" s="8"/>
       <x:c r="K52" s="8"/>
       <x:c r="L52" s="8"/>
       <x:c r="M52"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="8" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="B53" s="8" t="str">
-        <x:v>methodmesh_full_json</x:v>
-      </x:c>
-      <x:c r="C53" s="8" t="str">
-        <x:v>MethodMesh FULL JSON</x:v>
-      </x:c>
-      <x:c r="D53" s="8" t="str">
-        <x:v>Returned by MethodMesh.</x:v>
-      </x:c>
+      <x:c r="A53" s="8"/>
+      <x:c r="B53" s="8"/>
+      <x:c r="C53" s="8"/>
+      <x:c r="D53" s="8"/>
       <x:c r="E53" s="8"/>
       <x:c r="F53" s="8"/>
       <x:c r="G53" s="8"/>
       <x:c r="H53" s="8"/>
       <x:c r="I53" s="8"/>
-      <x:c r="J53" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+      <x:c r="J53" s="8"/>
       <x:c r="K53" s="8"/>
       <x:c r="L53" s="8"/>
       <x:c r="M53"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="8" t="str">
-        <x:v>end group</x:v>
-      </x:c>
-      <x:c r="B54" s="8" t="str">
-        <x:v>run_nfc_credential_provisioning_end</x:v>
-      </x:c>
+      <x:c r="A54" s="8"/>
+      <x:c r="B54" s="8"/>
       <x:c r="C54" s="8"/>
       <x:c r="D54" s="8"/>
       <x:c r="E54" s="8"/>
@@ -1612,22 +1308,12 @@
       <x:c r="M54"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="8" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="B55" s="8" t="str">
-        <x:v>provision_summary</x:v>
-      </x:c>
-      <x:c r="C55" s="8" t="str">
-        <x:v>Credential provisioning result</x:v>
-      </x:c>
-      <x:c r="D55" s="8" t="str">
-        <x:v>Credential ${credential_id}; MethodMesh status ${methodmesh_status}; write verified ${write_verified}; issuer ${issuer_key_id}; issuer fingerprint ${issuer_public_key_fingerprint_sha256}.</x:v>
-      </x:c>
+      <x:c r="A55" s="8"/>
+      <x:c r="B55" s="8"/>
+      <x:c r="C55" s="8"/>
+      <x:c r="D55" s="8"/>
       <x:c r="E55" s="8"/>
-      <x:c r="F55" s="8" t="str">
-        <x:v>${methodmesh_status} != ''</x:v>
-      </x:c>
+      <x:c r="F55" s="8"/>
       <x:c r="G55" s="8"/>
       <x:c r="H55" s="8"/>
       <x:c r="I55" s="8"/>
@@ -1637,18 +1323,10 @@
       <x:c r="M55"/>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="8" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="B56" s="8" t="str">
-        <x:v>registry_architecture_note</x:v>
-      </x:c>
-      <x:c r="C56" s="8" t="str">
-        <x:v>Registry record retained</x:v>
-      </x:c>
-      <x:c r="D56" s="8" t="str">
-        <x:v>Name, role, site, start/end dates, authorisation and issuance reason remain in the study credential registry and are linked to credential_id. The full issuer_public_key_fingerprint_sha256 is the canonical provisioning-device identity used later for central reconciliation. These governance fields are not silently added to the ROSC1 card.</x:v>
-      </x:c>
+      <x:c r="A56" s="8"/>
+      <x:c r="B56" s="8"/>
+      <x:c r="C56" s="8"/>
+      <x:c r="D56" s="8"/>
       <x:c r="E56" s="8"/>
       <x:c r="F56" s="8"/>
       <x:c r="G56" s="8"/>
@@ -4069,7 +3747,7 @@
         <x:v>nfc_credential_provisioning</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>2026092502</x:v>
+        <x:v>2026093006</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>English</x:v>

</xml_diff>

<commit_message>
Release v2.12.0: in-app NFC ODK compiler
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/nfc/example_odk_nfc_credential_provisioning.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/nfc/example_odk_nfc_credential_provisioning.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Ra8eee4f07ceb4088"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R34c2558039c04d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Re299aaf4d89c4bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rbe39e7d339614b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R365072cf3cbc4fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rb988b195a4d14186"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,7 +497,7 @@
       </x:c>
       <x:c r="K8" s="8"/>
       <x:c r="L8" s="8" t="str">
-        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_valid_until_date=${valid_until_date_iso},input_overwrite_policy=${overwrite_policy_input},input_payload_mode='FULL',return_mode='flat')</x:v>
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_nfc_form_contract_version='v1',input_nfc_method_version='1.0.1',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_valid_until_date=${valid_until_date_iso},input_overwrite_policy=${overwrite_policy_input},input_payload_mode='FULL',return_mode='flat')</x:v>
       </x:c>
       <x:c r="M8"/>
     </x:row>

</xml_diff>